<commit_message>
docs(tools): sync 120-tool catalog to 97 implemented
</commit_message>
<xml_diff>
--- a/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
+++ b/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R6b74cf95bc864973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="Rf86e72ea73364b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留25" sheetId="3" r:id="R836780b79dc543d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R6397c2d5789a4d75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R7a1d7a546c2f430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Reed149f87c814f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R93fab040d84b4860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留21" sheetId="3" r:id="R2b900303c3ad4411"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="Red9d995618dd4fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R0f5c5b4d8c384e4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>基线：main @ 04444df；P1-W12新增7项后已实现93项，既有86项实现保持原样。</x:v>
+        <x:v>基线：main @ 28630c0；P1-W13新增4项后已实现97项，既有93项实现保持原样。</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -536,14 +536,14 @@
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="18" t="str">
-        <x:v>当前已实现（不修改）</x:v>
+        <x:v>当前已实现（累计）</x:v>
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:f>COUNTIF('最终120路线'!$D$2:$D$121,"已实现")</x:f>
-        <x:v>93</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>1. 已实现93项不改代码、不改ID、不撤销资格；P1-W12只新增7项。</x:v>
+        <x:v>1. 已实现97项不改代码、不改ID、不撤销资格；P1-W13只新增4项。</x:v>
       </x:c>
       <x:c r="E6" s="27"/>
       <x:c r="F6" s="27"/>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:f>COUNTIFS('最终120路线'!$D$2:$D$121,"已实现",'最终120路线'!$G$2:$G$121,"是")</x:f>
-        <x:v>75</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
         <x:v>2. 延期项不注册、不生成空Schema、不计入count_eligible。</x:v>
@@ -572,7 +572,7 @@
       </x:c>
       <x:c r="B8" s="20" t="n">
         <x:f>120-B7</x:f>
-        <x:v>45</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>3. 后续工具不得以DS042、现场时序、企业标签或本地训练权重为准入前提。</x:v>
@@ -603,8 +603,8 @@
         <x:v>后续保留并去现场化</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:f>COUNTA('后续保留25'!$A$2:$A$26)</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTA('后续保留21'!$A$2:$A$22)</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D10" s="27" t="str">
         <x:v>5. 允许使用公开算法、批准数据库和仓库内版本化常数。</x:v>
@@ -636,7 +636,7 @@
       </x:c>
       <x:c r="B12" s="20" t="n">
         <x:f>B10+B11</x:f>
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
         <x:v>7. 任何未来恢复的现场模型必须另行完成数据授权、脱敏和时序验证。</x:v>
@@ -657,7 +657,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>计数闭合：93 已实现 + 25 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
+        <x:v>计数闭合：97 已实现 + 21 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
       </x:c>
       <x:c r="B15" s="31"/>
       <x:c r="C15" s="31"/>
@@ -1471,28 +1471,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="18" t="str">
-        <x:v>C008</x:v>
+        <x:v>E106</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
-        <x:v>C008</x:v>
+        <x:v>E006</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str">
-        <x:v>动力学与传递</x:v>
+        <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
-        <x:v>熔渣/钢液黏度估算</x:v>
+        <x:v>Rist操作线</x:v>
       </x:c>
       <x:c r="F2" s="18" t="str">
-        <x:v>版本化公开黏度关联式；首版不做机器学习回归</x:v>
+        <x:v>完整Rist操作线；新运行时ID E106，保留既有E006简化实现</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
-        <x:v>渣/钢组成、温度</x:v>
+        <x:v>炉料、顶煤气、燃料比、还原度</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
-        <x:v>黏度、置信区间</x:v>
+        <x:v>操作线、理想点、直接还原度</x:v>
       </x:c>
       <x:c r="I2" s="18" t="str">
-        <x:v>调用方显式提供组成、温度和关联式版本</x:v>
+        <x:v>显式炉料、顶煤气、燃料比和还原度</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
         <x:v>否</x:v>
@@ -1501,19 +1501,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L2" s="18" t="str">
-        <x:v>公开渣系/金属黏度经验关联式及其适用域</x:v>
+        <x:v>Rist操作线与C/O守恒</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>A004</x:v>
+        <x:v>E001-E005,E011</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
         <x:v>中</x:v>
       </x:c>
       <x:c r="O2" s="18" t="str">
-        <x:v>删除本地标定与训练路径</x:v>
+        <x:v>不修改既有E006；新增完整目录能力</x:v>
       </x:c>
       <x:c r="P2" s="18" t="str">
-        <x:v>estimate_melt_viscosity</x:v>
+        <x:v>calc_rist_operating_line</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1521,28 +1521,28 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="18" t="str">
-        <x:v>D018</x:v>
+        <x:v>E109</x:v>
       </x:c>
       <x:c r="C3" s="18" t="str">
-        <x:v>D018</x:v>
+        <x:v>E009</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
-        <x:v>转炉炼钢</x:v>
+        <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
-        <x:v>吹氧制度优化</x:v>
+        <x:v>喷煤等效替代</x:v>
       </x:c>
       <x:c r="F3" s="18" t="str">
-        <x:v>静态分段供氧约束优化；不读取炉气/喷溅时序</x:v>
+        <x:v>完整喷煤置换比能量/碳平衡；新运行时ID E109</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
-        <x:v>目标C/T/P、装料、设备约束</x:v>
+        <x:v>煤/焦性质、喷煤量、炉况</x:v>
       </x:c>
       <x:c r="H3" s="18" t="str">
-        <x:v>供氧曲线、枪位曲线、预计指标</x:v>
+        <x:v>等效焦炭替代量、边际收益</x:v>
       </x:c>
       <x:c r="I3" s="18" t="str">
-        <x:v>显式目标、装料、设备上下限和版本化规则</x:v>
+        <x:v>显式煤/焦工业分析、热值和工况边界</x:v>
       </x:c>
       <x:c r="J3" s="18" t="str">
         <x:v>否</x:v>
@@ -1551,19 +1551,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L3" s="18" t="str">
-        <x:v>物料/热平衡约束与确定性优化</x:v>
+        <x:v>固定碳、热值与风口区平衡</x:v>
       </x:c>
       <x:c r="M3" s="18" t="str">
-        <x:v>D002,D007,D016,G012</x:v>
+        <x:v>E003,E005,E007</x:v>
       </x:c>
       <x:c r="N3" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O3" s="18" t="str">
-        <x:v>降级为离线静态方案，不作在线控制</x:v>
+        <x:v>不修改既有E009范围变体</x:v>
       </x:c>
       <x:c r="P3" s="18" t="str">
-        <x:v>optimize_blowing_schedule</x:v>
+        <x:v>calc_pci_replacement_ratio</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" hidden="0" customHeight="1">
@@ -1571,28 +1571,28 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
-        <x:v>D019</x:v>
+        <x:v>E010</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>D019</x:v>
+        <x:v>E010</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
-        <x:v>转炉炼钢</x:v>
+        <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>合金加入优化</x:v>
+        <x:v>炉顶煤气组成</x:v>
       </x:c>
       <x:c r="F4" s="18" t="str">
-        <x:v>线性/混合整数最小成本配料</x:v>
+        <x:v>C/O/H/N平衡与反应平衡</x:v>
       </x:c>
       <x:c r="G4" s="18" t="str">
-        <x:v>钢水成分、目标规格、合金成分/价格/收得率</x:v>
+        <x:v>风量、燃料、还原度、湿分</x:v>
       </x:c>
       <x:c r="H4" s="18" t="str">
-        <x:v>合金加入方案、成本、约束余量</x:v>
+        <x:v>CO/CO2/H2/N2组成与体积</x:v>
       </x:c>
       <x:c r="I4" s="18" t="str">
-        <x:v>显式合金成分、价格、收得率与目标规格</x:v>
+        <x:v>显式风量、燃料、还原度和湿分</x:v>
       </x:c>
       <x:c r="J4" s="18" t="str">
         <x:v>否</x:v>
@@ -1601,19 +1601,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L4" s="18" t="str">
-        <x:v>线性/混合整数配料优化</x:v>
+        <x:v>C/O/H/N元素守恒与气相平衡</x:v>
       </x:c>
       <x:c r="M4" s="18" t="str">
-        <x:v>A004,D023,G012</x:v>
+        <x:v>E003-E005,E011,E012</x:v>
       </x:c>
       <x:c r="N4" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O4" s="18" t="str">
-        <x:v>收得率由调用方提供，不从历史炉次学习</x:v>
+        <x:v>输出理论煤气组成，不接在线分析仪</x:v>
       </x:c>
       <x:c r="P4" s="18" t="str">
-        <x:v>optimize_alloy_additions</x:v>
+        <x:v>calc_top_gas_composition</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" hidden="0" customHeight="1">
@@ -1621,28 +1621,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>D020</x:v>
+        <x:v>E013</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>D020</x:v>
+        <x:v>E013</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
-        <x:v>转炉炼钢</x:v>
+        <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>冷却剂/废钢加入优化</x:v>
+        <x:v>风口回旋区绝热火焰温度</x:v>
       </x:c>
       <x:c r="F5" s="18" t="str">
-        <x:v>热平衡约束下最小成本/最小波动优化</x:v>
+        <x:v>风口区绝热热平衡</x:v>
       </x:c>
       <x:c r="G5" s="18" t="str">
-        <x:v>热状态、废钢/矿石/冷却剂属性</x:v>
+        <x:v>风温、富氧、湿分、喷煤/气</x:v>
       </x:c>
       <x:c r="H5" s="18" t="str">
-        <x:v>加入量、终温区间、成本</x:v>
+        <x:v>RAFT、热量分项</x:v>
       </x:c>
       <x:c r="I5" s="18" t="str">
-        <x:v>显式热状态、物性、成本和设备约束</x:v>
+        <x:v>显式风温、富氧、湿分、喷吹燃料组成</x:v>
       </x:c>
       <x:c r="J5" s="18" t="str">
         <x:v>否</x:v>
@@ -1651,19 +1651,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L5" s="18" t="str">
-        <x:v>热平衡约束的确定性优化</x:v>
+        <x:v>风口回旋区绝热能量守恒</x:v>
       </x:c>
       <x:c r="M5" s="18" t="str">
-        <x:v>B003,D002,G012</x:v>
+        <x:v>B012,E012</x:v>
       </x:c>
       <x:c r="N5" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O5" s="18" t="str">
-        <x:v>不读取企业历史炉次</x:v>
+        <x:v>作为离线理论RAFT，不依赖风口传感器</x:v>
       </x:c>
       <x:c r="P5" s="18" t="str">
-        <x:v>optimize_coolant_scrap_addition</x:v>
+        <x:v>calc_raceway_adiabatic_flame_temp</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" hidden="0" customHeight="1">
@@ -1671,28 +1671,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>E106</x:v>
+        <x:v>E015</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>E006</x:v>
+        <x:v>E015</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
         <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>Rist操作线</x:v>
+        <x:v>透气性指数</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>完整Rist操作线；新运行时ID E106，保留既有E006简化实现</x:v>
+        <x:v>单工况透气性指数；删除趋势异常输出</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
-        <x:v>炉料、顶煤气、燃料比、还原度</x:v>
+        <x:v>压差、风量、炉顶压力、料线</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
-        <x:v>操作线、理想点、直接还原度</x:v>
+        <x:v>透气性指数、趋势异常</x:v>
       </x:c>
       <x:c r="I6" s="18" t="str">
-        <x:v>显式炉料、顶煤气、燃料比和还原度</x:v>
+        <x:v>调用方显式提供压差、风量、炉顶压力和料柱高度</x:v>
       </x:c>
       <x:c r="J6" s="18" t="str">
         <x:v>否</x:v>
@@ -1701,19 +1701,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L6" s="18" t="str">
-        <x:v>Rist操作线与C/O守恒</x:v>
+        <x:v>压差—流量归一化指数</x:v>
       </x:c>
       <x:c r="M6" s="18" t="str">
-        <x:v>E001-E005,E011</x:v>
+        <x:v>E014</x:v>
       </x:c>
       <x:c r="N6" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O6" s="18" t="str">
-        <x:v>不修改既有E006；新增完整目录能力</x:v>
+        <x:v>不读取连续时序；不提供炉况预警</x:v>
       </x:c>
       <x:c r="P6" s="18" t="str">
-        <x:v>calc_rist_operating_line</x:v>
+        <x:v>calc_permeability_index</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" hidden="0" customHeight="1">
@@ -1721,28 +1721,28 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="18" t="str">
-        <x:v>E109</x:v>
+        <x:v>E020</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>E009</x:v>
+        <x:v>E020</x:v>
       </x:c>
       <x:c r="D7" s="18" t="str">
         <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>喷煤等效替代</x:v>
+        <x:v>高炉碳足迹</x:v>
       </x:c>
       <x:c r="F7" s="18" t="str">
-        <x:v>完整喷煤置换比能量/碳平衡；新运行时ID E109</x:v>
+        <x:v>活动数据×排放因子；工序边界与分配规则</x:v>
       </x:c>
       <x:c r="G7" s="18" t="str">
-        <x:v>煤/焦性质、喷煤量、炉况</x:v>
+        <x:v>焦/煤/电/气/原料/产量、因子版本</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
-        <x:v>等效焦炭替代量、边际收益</x:v>
+        <x:v>tCO2e/tHM、分项排放、范围说明</x:v>
       </x:c>
       <x:c r="I7" s="18" t="str">
-        <x:v>显式煤/焦工业分析、热值和工况边界</x:v>
+        <x:v>调用方显式提供活动数据；排放因子使用公开版本化资产</x:v>
       </x:c>
       <x:c r="J7" s="18" t="str">
         <x:v>否</x:v>
@@ -1751,19 +1751,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L7" s="18" t="str">
-        <x:v>固定碳、热值与风口区平衡</x:v>
+        <x:v>ISO 14040/14044与GHG Protocol边界记录</x:v>
       </x:c>
       <x:c r="M7" s="18" t="str">
-        <x:v>E003,E005,E007</x:v>
+        <x:v>E001,E003,E005</x:v>
       </x:c>
       <x:c r="N7" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O7" s="18" t="str">
-        <x:v>不修改既有E009范围变体</x:v>
+        <x:v>不读取企业生产数据库</x:v>
       </x:c>
       <x:c r="P7" s="18" t="str">
-        <x:v>calc_pci_replacement_ratio</x:v>
+        <x:v>calc_bf_carbon_footprint</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" hidden="0" customHeight="1">
@@ -1771,28 +1771,28 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>E010</x:v>
+        <x:v>F008</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>E010</x:v>
+        <x:v>F008</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>炉顶煤气组成</x:v>
+        <x:v>二冷总水量计算</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>C/O/H/N平衡与反应平衡</x:v>
+        <x:v>目标表面温度/比水量经验模型</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
-        <x:v>风量、燃料、还原度、湿分</x:v>
+        <x:v>钢种、断面、拉速、目标温度</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
-        <x:v>CO/CO2/H2/N2组成与体积</x:v>
+        <x:v>总水量、比水量</x:v>
       </x:c>
       <x:c r="I8" s="18" t="str">
-        <x:v>显式风量、燃料、还原度和湿分</x:v>
+        <x:v>显式断面、拉速、目标热负荷/比水量参数</x:v>
       </x:c>
       <x:c r="J8" s="18" t="str">
         <x:v>否</x:v>
@@ -1801,19 +1801,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L8" s="18" t="str">
-        <x:v>C/O/H/N元素守恒与气相平衡</x:v>
+        <x:v>质量流量与比水量/热量平衡</x:v>
       </x:c>
       <x:c r="M8" s="18" t="str">
-        <x:v>E003-E005,E011,E012</x:v>
+        <x:v>F003,F005</x:v>
       </x:c>
       <x:c r="N8" s="18" t="str">
         <x:v>低</x:v>
       </x:c>
       <x:c r="O8" s="18" t="str">
-        <x:v>输出理论煤气组成，不接在线分析仪</x:v>
+        <x:v>不从历史浇次拟合参数</x:v>
       </x:c>
       <x:c r="P8" s="18" t="str">
-        <x:v>calc_top_gas_composition</x:v>
+        <x:v>calc_total_secondary_cooling_water</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" hidden="0" customHeight="1">
@@ -1821,28 +1821,28 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>E013</x:v>
+        <x:v>F009</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>E013</x:v>
+        <x:v>F009</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>风口回旋区绝热火焰温度</x:v>
+        <x:v>二冷分区水量分配</x:v>
       </x:c>
       <x:c r="F9" s="18" t="str">
-        <x:v>风口区绝热热平衡</x:v>
+        <x:v>各区换热模型+温度/回温约束</x:v>
       </x:c>
       <x:c r="G9" s="18" t="str">
-        <x:v>风温、富氧、湿分、喷煤/气</x:v>
+        <x:v>总水量、区段、喷嘴、拉速、目标温度</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
-        <x:v>RAFT、热量分项</x:v>
+        <x:v>分区水量、温度曲线、约束余量</x:v>
       </x:c>
       <x:c r="I9" s="18" t="str">
-        <x:v>显式风温、富氧、湿分、喷吹燃料组成</x:v>
+        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
       </x:c>
       <x:c r="J9" s="18" t="str">
         <x:v>否</x:v>
@@ -1851,19 +1851,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L9" s="18" t="str">
-        <x:v>风口回旋区绝热能量守恒</x:v>
+        <x:v>分区热平衡与约束优化</x:v>
       </x:c>
       <x:c r="M9" s="18" t="str">
-        <x:v>B012,E012</x:v>
+        <x:v>F005,F008,G012</x:v>
       </x:c>
       <x:c r="N9" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O9" s="18" t="str">
-        <x:v>作为离线理论RAFT，不依赖风口传感器</x:v>
+        <x:v>作为离线方案，不连接阀门或PLC</x:v>
       </x:c>
       <x:c r="P9" s="18" t="str">
-        <x:v>calc_raceway_adiabatic_flame_temp</x:v>
+        <x:v>allocate_secondary_cooling_water</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" hidden="0" customHeight="1">
@@ -1871,28 +1871,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>E015</x:v>
+        <x:v>F011</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>E015</x:v>
+        <x:v>F011</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>透气性指数</x:v>
+        <x:v>拉速优化</x:v>
       </x:c>
       <x:c r="F10" s="18" t="str">
-        <x:v>单工况透气性指数；删除趋势异常输出</x:v>
+        <x:v>产量、凝固终点、温度、质量风险多目标优化</x:v>
       </x:c>
       <x:c r="G10" s="18" t="str">
-        <x:v>压差、风量、炉顶压力、料线</x:v>
+        <x:v>钢种、断面、温度、水量、设备约束</x:v>
       </x:c>
       <x:c r="H10" s="18" t="str">
-        <x:v>透气性指数、趋势异常</x:v>
+        <x:v>拉速建议、风险/产量权衡</x:v>
       </x:c>
       <x:c r="I10" s="18" t="str">
-        <x:v>调用方显式提供压差、风量、炉顶压力和料柱高度</x:v>
+        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
       </x:c>
       <x:c r="J10" s="18" t="str">
         <x:v>否</x:v>
@@ -1901,19 +1901,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L10" s="18" t="str">
-        <x:v>压差—流量归一化指数</x:v>
+        <x:v>F005/F006物理约束下离线搜索</x:v>
       </x:c>
       <x:c r="M10" s="18" t="str">
-        <x:v>E014</x:v>
+        <x:v>F005,F006,F009,G012</x:v>
       </x:c>
       <x:c r="N10" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O10" s="18" t="str">
-        <x:v>不读取连续时序；不提供炉况预警</x:v>
+        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
       </x:c>
       <x:c r="P10" s="18" t="str">
-        <x:v>calc_permeability_index</x:v>
+        <x:v>optimize_casting_speed</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" hidden="0" customHeight="1">
@@ -1921,28 +1921,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
-        <x:v>E020</x:v>
+        <x:v>F014</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
-        <x:v>E020</x:v>
+        <x:v>F014</x:v>
       </x:c>
       <x:c r="D11" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>高炉碳足迹</x:v>
+        <x:v>铸坯热应力/应变</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
-        <x:v>活动数据×排放因子；工序边界与分配规则</x:v>
+        <x:v>温度场驱动热弹塑性/裂纹判据</x:v>
       </x:c>
       <x:c r="G11" s="18" t="str">
-        <x:v>焦/煤/电/气/原料/产量、因子版本</x:v>
+        <x:v>温度场、材料高温力学、边界条件</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
-        <x:v>tCO2e/tHM、分项排放、范围说明</x:v>
+        <x:v>应力/应变、危险位置</x:v>
       </x:c>
       <x:c r="I11" s="18" t="str">
-        <x:v>调用方显式提供活动数据；排放因子使用公开版本化资产</x:v>
+        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
       </x:c>
       <x:c r="J11" s="18" t="str">
         <x:v>否</x:v>
@@ -1951,19 +1951,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L11" s="18" t="str">
-        <x:v>ISO 14040/14044与GHG Protocol边界记录</x:v>
+        <x:v>热应变与简化弹塑性/有限元</x:v>
       </x:c>
       <x:c r="M11" s="18" t="str">
-        <x:v>E001,E003,E005</x:v>
+        <x:v>F005,G003</x:v>
       </x:c>
       <x:c r="N11" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O11" s="18" t="str">
-        <x:v>不读取企业生产数据库</x:v>
+        <x:v>不需要现场测温；仅分析显式温度场</x:v>
       </x:c>
       <x:c r="P11" s="18" t="str">
-        <x:v>calc_bf_carbon_footprint</x:v>
+        <x:v>calc_casting_thermal_stress</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" hidden="0" customHeight="1">
@@ -1971,28 +1971,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="18" t="str">
-        <x:v>F008</x:v>
+        <x:v>F018</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
-        <x:v>F008</x:v>
+        <x:v>F018</x:v>
       </x:c>
       <x:c r="D12" s="18" t="str">
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>二冷总水量计算</x:v>
+        <x:v>夹杂物上浮时间</x:v>
       </x:c>
       <x:c r="F12" s="18" t="str">
-        <x:v>目标表面温度/比水量经验模型</x:v>
+        <x:v>Stokes上浮+流场修正</x:v>
       </x:c>
       <x:c r="G12" s="18" t="str">
-        <x:v>钢种、断面、拉速、目标温度</x:v>
+        <x:v>夹杂尺寸/密度、钢液物性、流场尺度</x:v>
       </x:c>
       <x:c r="H12" s="18" t="str">
-        <x:v>总水量、比水量</x:v>
+        <x:v>上浮速度、停留时间、捕获概率</x:v>
       </x:c>
       <x:c r="I12" s="18" t="str">
-        <x:v>显式断面、拉速、目标热负荷/比水量参数</x:v>
+        <x:v>显式夹杂尺寸/密度、钢液物性和流动尺度</x:v>
       </x:c>
       <x:c r="J12" s="18" t="str">
         <x:v>否</x:v>
@@ -2001,19 +2001,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L12" s="18" t="str">
-        <x:v>质量流量与比水量/热量平衡</x:v>
+        <x:v>Stokes与阻力系数分段关联</x:v>
       </x:c>
       <x:c r="M12" s="18" t="str">
-        <x:v>F003,F005</x:v>
+        <x:v>C002,C010</x:v>
       </x:c>
       <x:c r="N12" s="18" t="str">
         <x:v>低</x:v>
       </x:c>
       <x:c r="O12" s="18" t="str">
-        <x:v>不从历史浇次拟合参数</x:v>
+        <x:v>不使用质量检测标签</x:v>
       </x:c>
       <x:c r="P12" s="18" t="str">
-        <x:v>calc_total_secondary_cooling_water</x:v>
+        <x:v>calc_inclusion_float_time</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" hidden="0" customHeight="1">
@@ -2021,28 +2021,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G003</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G003</x:v>
       </x:c>
       <x:c r="D13" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>二冷分区水量分配</x:v>
+        <x:v>一维传热PDE求解</x:v>
       </x:c>
       <x:c r="F13" s="18" t="str">
-        <x:v>各区换热模型+温度/回温约束</x:v>
+        <x:v>一维导热有限差分/有限体积</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
-        <x:v>总水量、区段、喷嘴、拉速、目标温度</x:v>
+        <x:v>几何、物性、热源、初边值</x:v>
       </x:c>
       <x:c r="H13" s="18" t="str">
-        <x:v>分区水量、温度曲线、约束余量</x:v>
+        <x:v>温度场、热流、能量闭合</x:v>
       </x:c>
       <x:c r="I13" s="18" t="str">
-        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
+        <x:v>显式几何、物性、热源和初边值</x:v>
       </x:c>
       <x:c r="J13" s="18" t="str">
         <x:v>否</x:v>
@@ -2051,19 +2051,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L13" s="18" t="str">
-        <x:v>分区热平衡与约束优化</x:v>
+        <x:v>一维导热有限差分/有限体积与能量闭合</x:v>
       </x:c>
       <x:c r="M13" s="18" t="str">
-        <x:v>F005,F008,G012</x:v>
+        <x:v>G001,G002,T001</x:v>
       </x:c>
       <x:c r="N13" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O13" s="18" t="str">
-        <x:v>作为离线方案，不连接阀门或PLC</x:v>
+        <x:v>纯数值PDE，不使用现场数据</x:v>
       </x:c>
       <x:c r="P13" s="18" t="str">
-        <x:v>allocate_secondary_cooling_water</x:v>
+        <x:v>solve_heat_pde_1d</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" hidden="0" customHeight="1">
@@ -2071,28 +2071,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="C14" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="D14" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>拉速优化</x:v>
+        <x:v>反应ODE求解</x:v>
       </x:c>
       <x:c r="F14" s="18" t="str">
-        <x:v>产量、凝固终点、温度、质量风险多目标优化</x:v>
+        <x:v>刚性/非刚性ODE自适应积分</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
-        <x:v>钢种、断面、温度、水量、设备约束</x:v>
+        <x:v>反应网络、速率、初值、时间区间</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
-        <x:v>拉速建议、风险/产量权衡</x:v>
+        <x:v>状态轨迹、事件、收敛信息</x:v>
       </x:c>
       <x:c r="I14" s="18" t="str">
-        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
+        <x:v>显式反应网络、速率表达式和初值</x:v>
       </x:c>
       <x:c r="J14" s="18" t="str">
         <x:v>否</x:v>
@@ -2101,19 +2101,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L14" s="18" t="str">
-        <x:v>F005/F006物理约束下离线搜索</x:v>
+        <x:v>自适应刚性/非刚性ODE积分</x:v>
       </x:c>
       <x:c r="M14" s="18" t="str">
-        <x:v>F005,F006,F009,G012</x:v>
+        <x:v>C001,G002</x:v>
       </x:c>
       <x:c r="N14" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O14" s="18" t="str">
-        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
+        <x:v>纯数值求解，不训练</x:v>
       </x:c>
       <x:c r="P14" s="18" t="str">
-        <x:v>optimize_casting_speed</x:v>
+        <x:v>solve_reaction_ode</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" hidden="0" customHeight="1">
@@ -2121,28 +2121,28 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>铸坯热应力/应变</x:v>
+        <x:v>CFD参数化案例生成</x:v>
       </x:c>
       <x:c r="F15" s="18" t="str">
-        <x:v>温度场驱动热弹塑性/裂纹判据</x:v>
+        <x:v>模板渲染+参数/边界条件校验</x:v>
       </x:c>
       <x:c r="G15" s="18" t="str">
-        <x:v>温度场、材料高温力学、边界条件</x:v>
+        <x:v>几何模板、物性、工况、求解器设置</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
-        <x:v>应力/应变、危险位置</x:v>
+        <x:v>可运行CFD案例目录、manifest</x:v>
       </x:c>
       <x:c r="I15" s="18" t="str">
-        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
+        <x:v>调用方显式提交几何模板、物性和工况</x:v>
       </x:c>
       <x:c r="J15" s="18" t="str">
         <x:v>否</x:v>
@@ -2151,19 +2151,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L15" s="18" t="str">
-        <x:v>热应变与简化弹塑性/有限元</x:v>
+        <x:v>OpenFOAM案例模板与schema校验</x:v>
       </x:c>
       <x:c r="M15" s="18" t="str">
-        <x:v>F005,G003</x:v>
+        <x:v>G001,G002,G013</x:v>
       </x:c>
       <x:c r="N15" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O15" s="18" t="str">
-        <x:v>不需要现场测温；仅分析显式温度场</x:v>
+        <x:v>DS042从必需来源中删除</x:v>
       </x:c>
       <x:c r="P15" s="18" t="str">
-        <x:v>calc_casting_thermal_stress</x:v>
+        <x:v>generate_cfd_case</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" hidden="0" customHeight="1">
@@ -2171,28 +2171,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="18" t="str">
-        <x:v>F018</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="C16" s="18" t="str">
-        <x:v>F018</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="D16" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>夹杂物上浮时间</x:v>
+        <x:v>参数化仿真批处理</x:v>
       </x:c>
       <x:c r="F16" s="18" t="str">
-        <x:v>Stokes上浮+流场修正</x:v>
+        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
       </x:c>
       <x:c r="G16" s="18" t="str">
-        <x:v>夹杂尺寸/密度、钢液物性、流场尺度</x:v>
+        <x:v>案例模板、参数空间、资源配额</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
-        <x:v>上浮速度、停留时间、捕获概率</x:v>
+        <x:v>运行状态、结果索引、失败原因</x:v>
       </x:c>
       <x:c r="I16" s="18" t="str">
-        <x:v>显式夹杂尺寸/密度、钢液物性和流动尺度</x:v>
+        <x:v>显式参数空间、案例模板和资源配额</x:v>
       </x:c>
       <x:c r="J16" s="18" t="str">
         <x:v>否</x:v>
@@ -2201,19 +2201,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L16" s="18" t="str">
-        <x:v>Stokes与阻力系数分段关联</x:v>
+        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
       </x:c>
       <x:c r="M16" s="18" t="str">
-        <x:v>C002,C010</x:v>
+        <x:v>G005,G013</x:v>
       </x:c>
       <x:c r="N16" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O16" s="18" t="str">
-        <x:v>不使用质量检测标签</x:v>
+        <x:v>不读取现场数据；只编排批准案例</x:v>
       </x:c>
       <x:c r="P16" s="18" t="str">
-        <x:v>calc_inclusion_float_time</x:v>
+        <x:v>run_parametric_simulation_batch</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" hidden="0" customHeight="1">
@@ -2221,28 +2221,28 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="C17" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="D17" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>一维传热PDE求解</x:v>
+        <x:v>插值与查表服务</x:v>
       </x:c>
       <x:c r="F17" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积</x:v>
+        <x:v>多维规则网格/散点插值+缓存</x:v>
       </x:c>
       <x:c r="G17" s="18" t="str">
-        <x:v>几何、物性、热源、初边值</x:v>
+        <x:v>查询点、表格版本、外推策略</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
-        <x:v>温度场、热流、能量闭合</x:v>
+        <x:v>插值值、距离、是否外推</x:v>
       </x:c>
       <x:c r="I17" s="18" t="str">
-        <x:v>显式几何、物性、热源和初边值</x:v>
+        <x:v>调用方上传或选择版本化查找表</x:v>
       </x:c>
       <x:c r="J17" s="18" t="str">
         <x:v>否</x:v>
@@ -2251,19 +2251,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L17" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积与能量闭合</x:v>
+        <x:v>规则网格/散点插值和外推距离</x:v>
       </x:c>
       <x:c r="M17" s="18" t="str">
-        <x:v>G001,G002,T001</x:v>
+        <x:v>A004</x:v>
       </x:c>
       <x:c r="N17" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O17" s="18" t="str">
-        <x:v>纯数值PDE，不使用现场数据</x:v>
+        <x:v>不连接企业实时表</x:v>
       </x:c>
       <x:c r="P17" s="18" t="str">
-        <x:v>solve_heat_pde_1d</x:v>
+        <x:v>interpolate_lookup_table</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" hidden="0" customHeight="1">
@@ -2271,28 +2271,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="C18" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="D18" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E18" s="18" t="str">
-        <x:v>反应ODE求解</x:v>
+        <x:v>敏感性分析</x:v>
       </x:c>
       <x:c r="F18" s="18" t="str">
-        <x:v>刚性/非刚性ODE自适应积分</x:v>
+        <x:v>局部导数、Morris/Sobol可选</x:v>
       </x:c>
       <x:c r="G18" s="18" t="str">
-        <x:v>反应网络、速率、初值、时间区间</x:v>
+        <x:v>模型、参数范围、采样预算</x:v>
       </x:c>
       <x:c r="H18" s="18" t="str">
-        <x:v>状态轨迹、事件、收敛信息</x:v>
+        <x:v>敏感度排序、交互效应</x:v>
       </x:c>
       <x:c r="I18" s="18" t="str">
-        <x:v>显式反应网络、速率表达式和初值</x:v>
+        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
       </x:c>
       <x:c r="J18" s="18" t="str">
         <x:v>否</x:v>
@@ -2301,19 +2301,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L18" s="18" t="str">
-        <x:v>自适应刚性/非刚性ODE积分</x:v>
+        <x:v>局部导数、Morris/Sobol</x:v>
       </x:c>
       <x:c r="M18" s="18" t="str">
-        <x:v>C001,G002</x:v>
+        <x:v>A010,G008</x:v>
       </x:c>
       <x:c r="N18" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O18" s="18" t="str">
-        <x:v>纯数值求解，不训练</x:v>
+        <x:v>离线分析，不使用历史成功率</x:v>
       </x:c>
       <x:c r="P18" s="18" t="str">
-        <x:v>solve_reaction_ode</x:v>
+        <x:v>run_sensitivity_analysis</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" hidden="0" customHeight="1">
@@ -2321,28 +2321,28 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="C19" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="D19" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>CFD参数化案例生成</x:v>
+        <x:v>Monte Carlo不确定度分析</x:v>
       </x:c>
       <x:c r="F19" s="18" t="str">
-        <x:v>模板渲染+参数/边界条件校验</x:v>
+        <x:v>输入分布采样+模型批量执行</x:v>
       </x:c>
       <x:c r="G19" s="18" t="str">
-        <x:v>几何模板、物性、工况、求解器设置</x:v>
+        <x:v>模型、输入分布、相关性、样本数</x:v>
       </x:c>
       <x:c r="H19" s="18" t="str">
-        <x:v>可运行CFD案例目录、manifest</x:v>
+        <x:v>输出分布、区间、失效概率</x:v>
       </x:c>
       <x:c r="I19" s="18" t="str">
-        <x:v>调用方显式提交几何模板、物性和工况</x:v>
+        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
       </x:c>
       <x:c r="J19" s="18" t="str">
         <x:v>否</x:v>
@@ -2351,19 +2351,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L19" s="18" t="str">
-        <x:v>OpenFOAM案例模板与schema校验</x:v>
+        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
       </x:c>
       <x:c r="M19" s="18" t="str">
-        <x:v>G001,G002,G013</x:v>
+        <x:v>A010,G006</x:v>
       </x:c>
       <x:c r="N19" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O19" s="18" t="str">
-        <x:v>DS042从必需来源中删除</x:v>
+        <x:v>离线不确定度分析</x:v>
       </x:c>
       <x:c r="P19" s="18" t="str">
-        <x:v>generate_cfd_case</x:v>
+        <x:v>run_monte_carlo_uncertainty</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" hidden="0" customHeight="1">
@@ -2371,28 +2371,28 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="C20" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="D20" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E20" s="18" t="str">
-        <x:v>参数化仿真批处理</x:v>
+        <x:v>贝叶斯优化</x:v>
       </x:c>
       <x:c r="F20" s="18" t="str">
-        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
+        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
       </x:c>
       <x:c r="G20" s="18" t="str">
-        <x:v>案例模板、参数空间、资源配额</x:v>
+        <x:v>目标函数、约束、变量范围、预算</x:v>
       </x:c>
       <x:c r="H20" s="18" t="str">
-        <x:v>运行状态、结果索引、失败原因</x:v>
+        <x:v>推荐下一组参数、最优历史、置信度</x:v>
       </x:c>
       <x:c r="I20" s="18" t="str">
-        <x:v>显式参数空间、案例模板和资源配额</x:v>
+        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
       </x:c>
       <x:c r="J20" s="18" t="str">
         <x:v>否</x:v>
@@ -2401,19 +2401,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L20" s="18" t="str">
-        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
+        <x:v>高斯过程/TPE采集函数</x:v>
       </x:c>
       <x:c r="M20" s="18" t="str">
-        <x:v>G005,G013</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N20" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O20" s="18" t="str">
-        <x:v>不读取现场数据；只编排批准案例</x:v>
+        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
       </x:c>
       <x:c r="P20" s="18" t="str">
-        <x:v>run_parametric_simulation_batch</x:v>
+        <x:v>run_bayesian_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" hidden="0" customHeight="1">
@@ -2421,28 +2421,28 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B21" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="C21" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="D21" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
-        <x:v>插值与查表服务</x:v>
+        <x:v>多目标优化</x:v>
       </x:c>
       <x:c r="F21" s="18" t="str">
-        <x:v>多维规则网格/散点插值+缓存</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="G21" s="18" t="str">
-        <x:v>查询点、表格版本、外推策略</x:v>
+        <x:v>目标、约束、变量、权重偏好</x:v>
       </x:c>
       <x:c r="H21" s="18" t="str">
-        <x:v>插值值、距离、是否外推</x:v>
+        <x:v>Pareto解集、折中解、约束状态</x:v>
       </x:c>
       <x:c r="I21" s="18" t="str">
-        <x:v>调用方上传或选择版本化查找表</x:v>
+        <x:v>显式目标、约束、变量范围和偏好</x:v>
       </x:c>
       <x:c r="J21" s="18" t="str">
         <x:v>否</x:v>
@@ -2451,19 +2451,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L21" s="18" t="str">
-        <x:v>规则网格/散点插值和外推距离</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="M21" s="18" t="str">
-        <x:v>A004</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N21" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O21" s="18" t="str">
-        <x:v>不连接企业实时表</x:v>
+        <x:v>不读取企业历史数据</x:v>
       </x:c>
       <x:c r="P21" s="18" t="str">
-        <x:v>interpolate_lookup_table</x:v>
+        <x:v>run_multiobjective_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" hidden="0" customHeight="1">
@@ -2471,28 +2471,28 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B22" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="C22" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="D22" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
-        <x:v>敏感性分析</x:v>
+        <x:v>约束规则校验器</x:v>
       </x:c>
       <x:c r="F22" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol可选</x:v>
+        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
       </x:c>
       <x:c r="G22" s="18" t="str">
-        <x:v>模型、参数范围、采样预算</x:v>
+        <x:v>模型输入输出、上下文、规则版本</x:v>
       </x:c>
       <x:c r="H22" s="18" t="str">
-        <x:v>敏感度排序、交互效应</x:v>
+        <x:v>通过/失败、违反规则、修复建议</x:v>
       </x:c>
       <x:c r="I22" s="18" t="str">
-        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
+        <x:v>显式模型输入输出与版本化JSON规则</x:v>
       </x:c>
       <x:c r="J22" s="18" t="str">
         <x:v>否</x:v>
@@ -2501,220 +2501,92 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L22" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol</x:v>
+        <x:v>表达式树、物料/能量与工艺边界</x:v>
       </x:c>
       <x:c r="M22" s="18" t="str">
-        <x:v>A010,G008</x:v>
+        <x:v>A005</x:v>
       </x:c>
       <x:c r="N22" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O22" s="18" t="str">
-        <x:v>离线分析，不使用历史成功率</x:v>
+        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
       </x:c>
       <x:c r="P22" s="18" t="str">
-        <x:v>run_sensitivity_analysis</x:v>
+        <x:v>validate_constraints</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" hidden="0" customHeight="1">
-      <x:c r="A23" s="18" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B23" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="C23" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="D23" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E23" s="18" t="str">
-        <x:v>Monte Carlo不确定度分析</x:v>
-      </x:c>
-      <x:c r="F23" s="18" t="str">
-        <x:v>输入分布采样+模型批量执行</x:v>
-      </x:c>
-      <x:c r="G23" s="18" t="str">
-        <x:v>模型、输入分布、相关性、样本数</x:v>
-      </x:c>
-      <x:c r="H23" s="18" t="str">
-        <x:v>输出分布、区间、失效概率</x:v>
-      </x:c>
-      <x:c r="I23" s="18" t="str">
-        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
-      </x:c>
-      <x:c r="J23" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K23" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L23" s="18" t="str">
-        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
-      </x:c>
-      <x:c r="M23" s="18" t="str">
-        <x:v>A010,G006</x:v>
-      </x:c>
-      <x:c r="N23" s="18" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="O23" s="18" t="str">
-        <x:v>离线不确定度分析</x:v>
-      </x:c>
-      <x:c r="P23" s="18" t="str">
-        <x:v>run_monte_carlo_uncertainty</x:v>
-      </x:c>
+      <x:c r="A23" s="18"/>
+      <x:c r="B23" s="18"/>
+      <x:c r="C23" s="18"/>
+      <x:c r="D23" s="18"/>
+      <x:c r="E23" s="18"/>
+      <x:c r="F23" s="18"/>
+      <x:c r="G23" s="18"/>
+      <x:c r="H23" s="18"/>
+      <x:c r="I23" s="18"/>
+      <x:c r="J23" s="18"/>
+      <x:c r="K23" s="18"/>
+      <x:c r="L23" s="18"/>
+      <x:c r="M23" s="18"/>
+      <x:c r="N23" s="18"/>
+      <x:c r="O23" s="18"/>
+      <x:c r="P23" s="18"/>
     </x:row>
     <x:row r="24" ht="42" hidden="0" customHeight="1">
-      <x:c r="A24" s="18" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B24" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="C24" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="D24" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E24" s="18" t="str">
-        <x:v>贝叶斯优化</x:v>
-      </x:c>
-      <x:c r="F24" s="18" t="str">
-        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
-      </x:c>
-      <x:c r="G24" s="18" t="str">
-        <x:v>目标函数、约束、变量范围、预算</x:v>
-      </x:c>
-      <x:c r="H24" s="18" t="str">
-        <x:v>推荐下一组参数、最优历史、置信度</x:v>
-      </x:c>
-      <x:c r="I24" s="18" t="str">
-        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
-      </x:c>
-      <x:c r="J24" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K24" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L24" s="18" t="str">
-        <x:v>高斯过程/TPE采集函数</x:v>
-      </x:c>
-      <x:c r="M24" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N24" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O24" s="18" t="str">
-        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
-      </x:c>
-      <x:c r="P24" s="18" t="str">
-        <x:v>run_bayesian_optimization</x:v>
-      </x:c>
+      <x:c r="A24" s="18"/>
+      <x:c r="B24" s="18"/>
+      <x:c r="C24" s="18"/>
+      <x:c r="D24" s="18"/>
+      <x:c r="E24" s="18"/>
+      <x:c r="F24" s="18"/>
+      <x:c r="G24" s="18"/>
+      <x:c r="H24" s="18"/>
+      <x:c r="I24" s="18"/>
+      <x:c r="J24" s="18"/>
+      <x:c r="K24" s="18"/>
+      <x:c r="L24" s="18"/>
+      <x:c r="M24" s="18"/>
+      <x:c r="N24" s="18"/>
+      <x:c r="O24" s="18"/>
+      <x:c r="P24" s="18"/>
     </x:row>
     <x:row r="25" ht="42" hidden="0" customHeight="1">
-      <x:c r="A25" s="18" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B25" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="C25" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="D25" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E25" s="18" t="str">
-        <x:v>多目标优化</x:v>
-      </x:c>
-      <x:c r="F25" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="G25" s="18" t="str">
-        <x:v>目标、约束、变量、权重偏好</x:v>
-      </x:c>
-      <x:c r="H25" s="18" t="str">
-        <x:v>Pareto解集、折中解、约束状态</x:v>
-      </x:c>
-      <x:c r="I25" s="18" t="str">
-        <x:v>显式目标、约束、变量范围和偏好</x:v>
-      </x:c>
-      <x:c r="J25" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K25" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L25" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="M25" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N25" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O25" s="18" t="str">
-        <x:v>不读取企业历史数据</x:v>
-      </x:c>
-      <x:c r="P25" s="18" t="str">
-        <x:v>run_multiobjective_optimization</x:v>
-      </x:c>
+      <x:c r="A25" s="18"/>
+      <x:c r="B25" s="18"/>
+      <x:c r="C25" s="18"/>
+      <x:c r="D25" s="18"/>
+      <x:c r="E25" s="18"/>
+      <x:c r="F25" s="18"/>
+      <x:c r="G25" s="18"/>
+      <x:c r="H25" s="18"/>
+      <x:c r="I25" s="18"/>
+      <x:c r="J25" s="18"/>
+      <x:c r="K25" s="18"/>
+      <x:c r="L25" s="18"/>
+      <x:c r="M25" s="18"/>
+      <x:c r="N25" s="18"/>
+      <x:c r="O25" s="18"/>
+      <x:c r="P25" s="18"/>
     </x:row>
     <x:row r="26" ht="42" hidden="0" customHeight="1">
-      <x:c r="A26" s="18" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B26" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="C26" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="D26" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E26" s="18" t="str">
-        <x:v>约束规则校验器</x:v>
-      </x:c>
-      <x:c r="F26" s="18" t="str">
-        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="G26" s="18" t="str">
-        <x:v>模型输入输出、上下文、规则版本</x:v>
-      </x:c>
-      <x:c r="H26" s="18" t="str">
-        <x:v>通过/失败、违反规则、修复建议</x:v>
-      </x:c>
-      <x:c r="I26" s="18" t="str">
-        <x:v>显式模型输入输出与版本化JSON规则</x:v>
-      </x:c>
-      <x:c r="J26" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K26" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L26" s="18" t="str">
-        <x:v>表达式树、物料/能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="M26" s="18" t="str">
-        <x:v>A005</x:v>
-      </x:c>
-      <x:c r="N26" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O26" s="18" t="str">
-        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
-      </x:c>
-      <x:c r="P26" s="18" t="str">
-        <x:v>validate_constraints</x:v>
-      </x:c>
+      <x:c r="A26" s="18"/>
+      <x:c r="B26" s="18"/>
+      <x:c r="C26" s="18"/>
+      <x:c r="D26" s="18"/>
+      <x:c r="E26" s="18"/>
+      <x:c r="F26" s="18"/>
+      <x:c r="G26" s="18"/>
+      <x:c r="H26" s="18"/>
+      <x:c r="I26" s="18"/>
+      <x:c r="J26" s="18"/>
+      <x:c r="K26" s="18"/>
+      <x:c r="L26" s="18"/>
+      <x:c r="M26" s="18"/>
+      <x:c r="N26" s="18"/>
+      <x:c r="O26" s="18"/>
+      <x:c r="P26" s="18"/>
     </x:row>
     <x:row r="27" ht="42" hidden="0" customHeight="1">
       <x:c r="A27"/>
@@ -7111,13 +6983,13 @@
         <x:v>C008</x:v>
       </x:c>
       <x:c r="C83" s="18" t="str">
-        <x:v>熔渣/钢液黏度估算</x:v>
+        <x:v>熔渣/液态金属黏度估算</x:v>
       </x:c>
       <x:c r="D83" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E83" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W13</x:v>
       </x:c>
       <x:c r="F83" s="18" t="str">
         <x:v>C008</x:v>
@@ -7129,7 +7001,7 @@
         <x:v>动力学与传递</x:v>
       </x:c>
       <x:c r="I83" s="18" t="str">
-        <x:v>调用方显式提供组成、温度和关联式版本</x:v>
+        <x:v>数据库版本化Urbain/Hirai关联式；调用方显式输入组成/物性</x:v>
       </x:c>
       <x:c r="J83" s="18" t="str">
         <x:v>否</x:v>
@@ -7138,10 +7010,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L83" s="18" t="str">
-        <x:v>planned.c008.v1</x:v>
+        <x:v>metallurgy.catalog.c008.melt_viscosity.v1</x:v>
       </x:c>
       <x:c r="M83" s="18" t="str">
-        <x:v>删除本地标定与训练路径</x:v>
+        <x:v>same</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="42" hidden="0" customHeight="1">
@@ -7152,13 +7024,13 @@
         <x:v>D018</x:v>
       </x:c>
       <x:c r="C84" s="18" t="str">
-        <x:v>吹氧制度优化</x:v>
+        <x:v>BOF静态分段供氧制度优化</x:v>
       </x:c>
       <x:c r="D84" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E84" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W13</x:v>
       </x:c>
       <x:c r="F84" s="18" t="str">
         <x:v>D018</x:v>
@@ -7170,7 +7042,7 @@
         <x:v>转炉炼钢</x:v>
       </x:c>
       <x:c r="I84" s="18" t="str">
-        <x:v>显式目标、装料、设备上下限和版本化规则</x:v>
+        <x:v>调用方显式提供总氧量、阶段边界/流量/枪位；静态LP</x:v>
       </x:c>
       <x:c r="J84" s="18" t="str">
         <x:v>否</x:v>
@@ -7179,10 +7051,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L84" s="18" t="str">
-        <x:v>planned.d018.v1</x:v>
+        <x:v>metallurgy.catalog.d018.bof_blowing_schedule_optimization.v1</x:v>
       </x:c>
       <x:c r="M84" s="18" t="str">
-        <x:v>降级为离线静态方案，不作在线控制</x:v>
+        <x:v>same</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="42" hidden="0" customHeight="1">
@@ -7193,13 +7065,13 @@
         <x:v>D019</x:v>
       </x:c>
       <x:c r="C85" s="18" t="str">
-        <x:v>合金加入优化</x:v>
+        <x:v>多合金最小成本补加优化</x:v>
       </x:c>
       <x:c r="D85" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E85" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W13</x:v>
       </x:c>
       <x:c r="F85" s="18" t="str">
         <x:v>D019</x:v>
@@ -7211,7 +7083,7 @@
         <x:v>转炉炼钢</x:v>
       </x:c>
       <x:c r="I85" s="18" t="str">
-        <x:v>显式合金成分、价格、收得率与目标规格</x:v>
+        <x:v>调用方显式提供钢液/目标/合金/成本/收得率；LP/MILP</x:v>
       </x:c>
       <x:c r="J85" s="18" t="str">
         <x:v>否</x:v>
@@ -7220,10 +7092,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L85" s="18" t="str">
-        <x:v>planned.d019.v1</x:v>
+        <x:v>metallurgy.catalog.d019.alloy_addition_optimization.v1</x:v>
       </x:c>
       <x:c r="M85" s="18" t="str">
-        <x:v>收得率由调用方提供，不从历史炉次学习</x:v>
+        <x:v>same</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="42" hidden="0" customHeight="1">
@@ -7234,13 +7106,13 @@
         <x:v>D020</x:v>
       </x:c>
       <x:c r="C86" s="18" t="str">
-        <x:v>冷却剂/废钢加入优化</x:v>
+        <x:v>冷却剂/废钢静态加入优化</x:v>
       </x:c>
       <x:c r="D86" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E86" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W13</x:v>
       </x:c>
       <x:c r="F86" s="18" t="str">
         <x:v>D020</x:v>
@@ -7252,7 +7124,7 @@
         <x:v>转炉炼钢</x:v>
       </x:c>
       <x:c r="I86" s="18" t="str">
-        <x:v>显式热状态、物性、成本和设备约束</x:v>
+        <x:v>调用方显式提供热状态/材料冷却能力/成本；LP/MILP</x:v>
       </x:c>
       <x:c r="J86" s="18" t="str">
         <x:v>否</x:v>
@@ -7261,10 +7133,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L86" s="18" t="str">
-        <x:v>planned.d020.v1</x:v>
+        <x:v>metallurgy.catalog.d020.coolant_scrap_optimization.v1</x:v>
       </x:c>
       <x:c r="M86" s="18" t="str">
-        <x:v>不读取企业历史炉次</x:v>
+        <x:v>same</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="42" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
docs(tools): sync 120-tool catalog to 101 implemented
</commit_message>
<xml_diff>
--- a/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
+++ b/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Reed149f87c814f02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R93fab040d84b4860"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留21" sheetId="3" r:id="R2b900303c3ad4411"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="Red9d995618dd4fc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R0f5c5b4d8c384e4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Re4b119dcd6514a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R9d1b3c690f7046d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留17" sheetId="3" r:id="Re38b9a8665a549b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="Rbca693d69f854281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="Rbeefa90f772043d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>基线：main @ 28630c0；P1-W13新增4项后已实现97项，既有93项实现保持原样。</x:v>
+        <x:v>基线：main @ 2028237；P1-W14新增4项后已实现101项，既有97项实现保持原样。</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -540,10 +540,10 @@
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:f>COUNTIF('最终120路线'!$D$2:$D$121,"已实现")</x:f>
-        <x:v>97</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>1. 已实现97项不改代码、不改ID、不撤销资格；P1-W13只新增4项。</x:v>
+        <x:v>已实现101项不改ID、不撤销资格；P1-W14新增E106、E109、E010、E013共4项。</x:v>
       </x:c>
       <x:c r="E6" s="27"/>
       <x:c r="F6" s="27"/>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:f>COUNTIFS('最终120路线'!$D$2:$D$121,"已实现",'最终120路线'!$G$2:$G$121,"是")</x:f>
-        <x:v>79</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
         <x:v>2. 延期项不注册、不生成空Schema、不计入count_eligible。</x:v>
@@ -572,7 +572,7 @@
       </x:c>
       <x:c r="B8" s="20" t="n">
         <x:f>120-B7</x:f>
-        <x:v>41</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>3. 后续工具不得以DS042、现场时序、企业标签或本地训练权重为准入前提。</x:v>
@@ -603,8 +603,8 @@
         <x:v>后续保留并去现场化</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:f>COUNTA('后续保留21'!$A$2:$A$22)</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTA('后续保留17'!$A$2:$A$18)</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D10" s="27" t="str">
         <x:v>5. 允许使用公开算法、批准数据库和仓库内版本化常数。</x:v>
@@ -636,7 +636,7 @@
       </x:c>
       <x:c r="B12" s="20" t="n">
         <x:f>B10+B11</x:f>
-        <x:v>23</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
         <x:v>7. 任何未来恢复的现场模型必须另行完成数据授权、脱敏和时序验证。</x:v>
@@ -657,7 +657,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>计数闭合：97 已实现 + 21 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
+        <x:v>计数闭合：101 已实现 + 17 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
       </x:c>
       <x:c r="B15" s="31"/>
       <x:c r="C15" s="31"/>
@@ -1471,28 +1471,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="18" t="str">
-        <x:v>E106</x:v>
+        <x:v>E015</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
-        <x:v>E006</x:v>
+        <x:v>E015</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str">
         <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
-        <x:v>Rist操作线</x:v>
+        <x:v>透气性指数</x:v>
       </x:c>
       <x:c r="F2" s="18" t="str">
-        <x:v>完整Rist操作线；新运行时ID E106，保留既有E006简化实现</x:v>
+        <x:v>单工况透气性指数；删除趋势异常输出</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
-        <x:v>炉料、顶煤气、燃料比、还原度</x:v>
+        <x:v>压差、风量、炉顶压力、料线</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
-        <x:v>操作线、理想点、直接还原度</x:v>
+        <x:v>透气性指数、趋势异常</x:v>
       </x:c>
       <x:c r="I2" s="18" t="str">
-        <x:v>显式炉料、顶煤气、燃料比和还原度</x:v>
+        <x:v>调用方显式提供压差、风量、炉顶压力和料柱高度</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
         <x:v>否</x:v>
@@ -1501,19 +1501,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L2" s="18" t="str">
-        <x:v>Rist操作线与C/O守恒</x:v>
+        <x:v>压差—流量归一化指数</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>E001-E005,E011</x:v>
+        <x:v>E014</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O2" s="18" t="str">
-        <x:v>不修改既有E006；新增完整目录能力</x:v>
+        <x:v>不读取连续时序；不提供炉况预警</x:v>
       </x:c>
       <x:c r="P2" s="18" t="str">
-        <x:v>calc_rist_operating_line</x:v>
+        <x:v>calc_permeability_index</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1521,28 +1521,28 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="18" t="str">
-        <x:v>E109</x:v>
+        <x:v>E020</x:v>
       </x:c>
       <x:c r="C3" s="18" t="str">
-        <x:v>E009</x:v>
+        <x:v>E020</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
         <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
-        <x:v>喷煤等效替代</x:v>
+        <x:v>高炉碳足迹</x:v>
       </x:c>
       <x:c r="F3" s="18" t="str">
-        <x:v>完整喷煤置换比能量/碳平衡；新运行时ID E109</x:v>
+        <x:v>活动数据×排放因子；工序边界与分配规则</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
-        <x:v>煤/焦性质、喷煤量、炉况</x:v>
+        <x:v>焦/煤/电/气/原料/产量、因子版本</x:v>
       </x:c>
       <x:c r="H3" s="18" t="str">
-        <x:v>等效焦炭替代量、边际收益</x:v>
+        <x:v>tCO2e/tHM、分项排放、范围说明</x:v>
       </x:c>
       <x:c r="I3" s="18" t="str">
-        <x:v>显式煤/焦工业分析、热值和工况边界</x:v>
+        <x:v>调用方显式提供活动数据；排放因子使用公开版本化资产</x:v>
       </x:c>
       <x:c r="J3" s="18" t="str">
         <x:v>否</x:v>
@@ -1551,19 +1551,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L3" s="18" t="str">
-        <x:v>固定碳、热值与风口区平衡</x:v>
+        <x:v>ISO 14040/14044与GHG Protocol边界记录</x:v>
       </x:c>
       <x:c r="M3" s="18" t="str">
-        <x:v>E003,E005,E007</x:v>
+        <x:v>E001,E003,E005</x:v>
       </x:c>
       <x:c r="N3" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O3" s="18" t="str">
-        <x:v>不修改既有E009范围变体</x:v>
+        <x:v>不读取企业生产数据库</x:v>
       </x:c>
       <x:c r="P3" s="18" t="str">
-        <x:v>calc_pci_replacement_ratio</x:v>
+        <x:v>calc_bf_carbon_footprint</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" hidden="0" customHeight="1">
@@ -1571,28 +1571,28 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
-        <x:v>E010</x:v>
+        <x:v>F008</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>E010</x:v>
+        <x:v>F008</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>炉顶煤气组成</x:v>
+        <x:v>二冷总水量计算</x:v>
       </x:c>
       <x:c r="F4" s="18" t="str">
-        <x:v>C/O/H/N平衡与反应平衡</x:v>
+        <x:v>目标表面温度/比水量经验模型</x:v>
       </x:c>
       <x:c r="G4" s="18" t="str">
-        <x:v>风量、燃料、还原度、湿分</x:v>
+        <x:v>钢种、断面、拉速、目标温度</x:v>
       </x:c>
       <x:c r="H4" s="18" t="str">
-        <x:v>CO/CO2/H2/N2组成与体积</x:v>
+        <x:v>总水量、比水量</x:v>
       </x:c>
       <x:c r="I4" s="18" t="str">
-        <x:v>显式风量、燃料、还原度和湿分</x:v>
+        <x:v>显式断面、拉速、目标热负荷/比水量参数</x:v>
       </x:c>
       <x:c r="J4" s="18" t="str">
         <x:v>否</x:v>
@@ -1601,19 +1601,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L4" s="18" t="str">
-        <x:v>C/O/H/N元素守恒与气相平衡</x:v>
+        <x:v>质量流量与比水量/热量平衡</x:v>
       </x:c>
       <x:c r="M4" s="18" t="str">
-        <x:v>E003-E005,E011,E012</x:v>
+        <x:v>F003,F005</x:v>
       </x:c>
       <x:c r="N4" s="18" t="str">
         <x:v>低</x:v>
       </x:c>
       <x:c r="O4" s="18" t="str">
-        <x:v>输出理论煤气组成，不接在线分析仪</x:v>
+        <x:v>不从历史浇次拟合参数</x:v>
       </x:c>
       <x:c r="P4" s="18" t="str">
-        <x:v>calc_top_gas_composition</x:v>
+        <x:v>calc_total_secondary_cooling_water</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" hidden="0" customHeight="1">
@@ -1621,28 +1621,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>E013</x:v>
+        <x:v>F009</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>E013</x:v>
+        <x:v>F009</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>风口回旋区绝热火焰温度</x:v>
+        <x:v>二冷分区水量分配</x:v>
       </x:c>
       <x:c r="F5" s="18" t="str">
-        <x:v>风口区绝热热平衡</x:v>
+        <x:v>各区换热模型+温度/回温约束</x:v>
       </x:c>
       <x:c r="G5" s="18" t="str">
-        <x:v>风温、富氧、湿分、喷煤/气</x:v>
+        <x:v>总水量、区段、喷嘴、拉速、目标温度</x:v>
       </x:c>
       <x:c r="H5" s="18" t="str">
-        <x:v>RAFT、热量分项</x:v>
+        <x:v>分区水量、温度曲线、约束余量</x:v>
       </x:c>
       <x:c r="I5" s="18" t="str">
-        <x:v>显式风温、富氧、湿分、喷吹燃料组成</x:v>
+        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
       </x:c>
       <x:c r="J5" s="18" t="str">
         <x:v>否</x:v>
@@ -1651,19 +1651,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L5" s="18" t="str">
-        <x:v>风口回旋区绝热能量守恒</x:v>
+        <x:v>分区热平衡与约束优化</x:v>
       </x:c>
       <x:c r="M5" s="18" t="str">
-        <x:v>B012,E012</x:v>
+        <x:v>F005,F008,G012</x:v>
       </x:c>
       <x:c r="N5" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O5" s="18" t="str">
-        <x:v>作为离线理论RAFT，不依赖风口传感器</x:v>
+        <x:v>作为离线方案，不连接阀门或PLC</x:v>
       </x:c>
       <x:c r="P5" s="18" t="str">
-        <x:v>calc_raceway_adiabatic_flame_temp</x:v>
+        <x:v>allocate_secondary_cooling_water</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" hidden="0" customHeight="1">
@@ -1671,28 +1671,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>E015</x:v>
+        <x:v>F011</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>E015</x:v>
+        <x:v>F011</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>透气性指数</x:v>
+        <x:v>拉速优化</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>单工况透气性指数；删除趋势异常输出</x:v>
+        <x:v>产量、凝固终点、温度、质量风险多目标优化</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
-        <x:v>压差、风量、炉顶压力、料线</x:v>
+        <x:v>钢种、断面、温度、水量、设备约束</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
-        <x:v>透气性指数、趋势异常</x:v>
+        <x:v>拉速建议、风险/产量权衡</x:v>
       </x:c>
       <x:c r="I6" s="18" t="str">
-        <x:v>调用方显式提供压差、风量、炉顶压力和料柱高度</x:v>
+        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
       </x:c>
       <x:c r="J6" s="18" t="str">
         <x:v>否</x:v>
@@ -1701,19 +1701,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L6" s="18" t="str">
-        <x:v>压差—流量归一化指数</x:v>
+        <x:v>F005/F006物理约束下离线搜索</x:v>
       </x:c>
       <x:c r="M6" s="18" t="str">
-        <x:v>E014</x:v>
+        <x:v>F005,F006,F009,G012</x:v>
       </x:c>
       <x:c r="N6" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O6" s="18" t="str">
-        <x:v>不读取连续时序；不提供炉况预警</x:v>
+        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
       </x:c>
       <x:c r="P6" s="18" t="str">
-        <x:v>calc_permeability_index</x:v>
+        <x:v>optimize_casting_speed</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" hidden="0" customHeight="1">
@@ -1721,28 +1721,28 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="18" t="str">
-        <x:v>E020</x:v>
+        <x:v>F014</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>E020</x:v>
+        <x:v>F014</x:v>
       </x:c>
       <x:c r="D7" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>高炉碳足迹</x:v>
+        <x:v>铸坯热应力/应变</x:v>
       </x:c>
       <x:c r="F7" s="18" t="str">
-        <x:v>活动数据×排放因子；工序边界与分配规则</x:v>
+        <x:v>温度场驱动热弹塑性/裂纹判据</x:v>
       </x:c>
       <x:c r="G7" s="18" t="str">
-        <x:v>焦/煤/电/气/原料/产量、因子版本</x:v>
+        <x:v>温度场、材料高温力学、边界条件</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
-        <x:v>tCO2e/tHM、分项排放、范围说明</x:v>
+        <x:v>应力/应变、危险位置</x:v>
       </x:c>
       <x:c r="I7" s="18" t="str">
-        <x:v>调用方显式提供活动数据；排放因子使用公开版本化资产</x:v>
+        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
       </x:c>
       <x:c r="J7" s="18" t="str">
         <x:v>否</x:v>
@@ -1751,19 +1751,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L7" s="18" t="str">
-        <x:v>ISO 14040/14044与GHG Protocol边界记录</x:v>
+        <x:v>热应变与简化弹塑性/有限元</x:v>
       </x:c>
       <x:c r="M7" s="18" t="str">
-        <x:v>E001,E003,E005</x:v>
+        <x:v>F005,G003</x:v>
       </x:c>
       <x:c r="N7" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O7" s="18" t="str">
-        <x:v>不读取企业生产数据库</x:v>
+        <x:v>不需要现场测温；仅分析显式温度场</x:v>
       </x:c>
       <x:c r="P7" s="18" t="str">
-        <x:v>calc_bf_carbon_footprint</x:v>
+        <x:v>calc_casting_thermal_stress</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" hidden="0" customHeight="1">
@@ -1771,28 +1771,28 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>F008</x:v>
+        <x:v>F018</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>F008</x:v>
+        <x:v>F018</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>二冷总水量计算</x:v>
+        <x:v>夹杂物上浮时间</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>目标表面温度/比水量经验模型</x:v>
+        <x:v>Stokes上浮+流场修正</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
-        <x:v>钢种、断面、拉速、目标温度</x:v>
+        <x:v>夹杂尺寸/密度、钢液物性、流场尺度</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
-        <x:v>总水量、比水量</x:v>
+        <x:v>上浮速度、停留时间、捕获概率</x:v>
       </x:c>
       <x:c r="I8" s="18" t="str">
-        <x:v>显式断面、拉速、目标热负荷/比水量参数</x:v>
+        <x:v>显式夹杂尺寸/密度、钢液物性和流动尺度</x:v>
       </x:c>
       <x:c r="J8" s="18" t="str">
         <x:v>否</x:v>
@@ -1801,19 +1801,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L8" s="18" t="str">
-        <x:v>质量流量与比水量/热量平衡</x:v>
+        <x:v>Stokes与阻力系数分段关联</x:v>
       </x:c>
       <x:c r="M8" s="18" t="str">
-        <x:v>F003,F005</x:v>
+        <x:v>C002,C010</x:v>
       </x:c>
       <x:c r="N8" s="18" t="str">
         <x:v>低</x:v>
       </x:c>
       <x:c r="O8" s="18" t="str">
-        <x:v>不从历史浇次拟合参数</x:v>
+        <x:v>不使用质量检测标签</x:v>
       </x:c>
       <x:c r="P8" s="18" t="str">
-        <x:v>calc_total_secondary_cooling_water</x:v>
+        <x:v>calc_inclusion_float_time</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" hidden="0" customHeight="1">
@@ -1821,28 +1821,28 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G003</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G003</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>二冷分区水量分配</x:v>
+        <x:v>一维传热PDE求解</x:v>
       </x:c>
       <x:c r="F9" s="18" t="str">
-        <x:v>各区换热模型+温度/回温约束</x:v>
+        <x:v>一维导热有限差分/有限体积</x:v>
       </x:c>
       <x:c r="G9" s="18" t="str">
-        <x:v>总水量、区段、喷嘴、拉速、目标温度</x:v>
+        <x:v>几何、物性、热源、初边值</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
-        <x:v>分区水量、温度曲线、约束余量</x:v>
+        <x:v>温度场、热流、能量闭合</x:v>
       </x:c>
       <x:c r="I9" s="18" t="str">
-        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
+        <x:v>显式几何、物性、热源和初边值</x:v>
       </x:c>
       <x:c r="J9" s="18" t="str">
         <x:v>否</x:v>
@@ -1851,19 +1851,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L9" s="18" t="str">
-        <x:v>分区热平衡与约束优化</x:v>
+        <x:v>一维导热有限差分/有限体积与能量闭合</x:v>
       </x:c>
       <x:c r="M9" s="18" t="str">
-        <x:v>F005,F008,G012</x:v>
+        <x:v>G001,G002,T001</x:v>
       </x:c>
       <x:c r="N9" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O9" s="18" t="str">
-        <x:v>作为离线方案，不连接阀门或PLC</x:v>
+        <x:v>纯数值PDE，不使用现场数据</x:v>
       </x:c>
       <x:c r="P9" s="18" t="str">
-        <x:v>allocate_secondary_cooling_water</x:v>
+        <x:v>solve_heat_pde_1d</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" hidden="0" customHeight="1">
@@ -1871,28 +1871,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>拉速优化</x:v>
+        <x:v>反应ODE求解</x:v>
       </x:c>
       <x:c r="F10" s="18" t="str">
-        <x:v>产量、凝固终点、温度、质量风险多目标优化</x:v>
+        <x:v>刚性/非刚性ODE自适应积分</x:v>
       </x:c>
       <x:c r="G10" s="18" t="str">
-        <x:v>钢种、断面、温度、水量、设备约束</x:v>
+        <x:v>反应网络、速率、初值、时间区间</x:v>
       </x:c>
       <x:c r="H10" s="18" t="str">
-        <x:v>拉速建议、风险/产量权衡</x:v>
+        <x:v>状态轨迹、事件、收敛信息</x:v>
       </x:c>
       <x:c r="I10" s="18" t="str">
-        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
+        <x:v>显式反应网络、速率表达式和初值</x:v>
       </x:c>
       <x:c r="J10" s="18" t="str">
         <x:v>否</x:v>
@@ -1901,19 +1901,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L10" s="18" t="str">
-        <x:v>F005/F006物理约束下离线搜索</x:v>
+        <x:v>自适应刚性/非刚性ODE积分</x:v>
       </x:c>
       <x:c r="M10" s="18" t="str">
-        <x:v>F005,F006,F009,G012</x:v>
+        <x:v>C001,G002</x:v>
       </x:c>
       <x:c r="N10" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O10" s="18" t="str">
-        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
+        <x:v>纯数值求解，不训练</x:v>
       </x:c>
       <x:c r="P10" s="18" t="str">
-        <x:v>optimize_casting_speed</x:v>
+        <x:v>solve_reaction_ode</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" hidden="0" customHeight="1">
@@ -1921,28 +1921,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="D11" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>铸坯热应力/应变</x:v>
+        <x:v>CFD参数化案例生成</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
-        <x:v>温度场驱动热弹塑性/裂纹判据</x:v>
+        <x:v>模板渲染+参数/边界条件校验</x:v>
       </x:c>
       <x:c r="G11" s="18" t="str">
-        <x:v>温度场、材料高温力学、边界条件</x:v>
+        <x:v>几何模板、物性、工况、求解器设置</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
-        <x:v>应力/应变、危险位置</x:v>
+        <x:v>可运行CFD案例目录、manifest</x:v>
       </x:c>
       <x:c r="I11" s="18" t="str">
-        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
+        <x:v>调用方显式提交几何模板、物性和工况</x:v>
       </x:c>
       <x:c r="J11" s="18" t="str">
         <x:v>否</x:v>
@@ -1951,19 +1951,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L11" s="18" t="str">
-        <x:v>热应变与简化弹塑性/有限元</x:v>
+        <x:v>OpenFOAM案例模板与schema校验</x:v>
       </x:c>
       <x:c r="M11" s="18" t="str">
-        <x:v>F005,G003</x:v>
+        <x:v>G001,G002,G013</x:v>
       </x:c>
       <x:c r="N11" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O11" s="18" t="str">
-        <x:v>不需要现场测温；仅分析显式温度场</x:v>
+        <x:v>DS042从必需来源中删除</x:v>
       </x:c>
       <x:c r="P11" s="18" t="str">
-        <x:v>calc_casting_thermal_stress</x:v>
+        <x:v>generate_cfd_case</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" hidden="0" customHeight="1">
@@ -1971,28 +1971,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="18" t="str">
-        <x:v>F018</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
-        <x:v>F018</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="D12" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>夹杂物上浮时间</x:v>
+        <x:v>参数化仿真批处理</x:v>
       </x:c>
       <x:c r="F12" s="18" t="str">
-        <x:v>Stokes上浮+流场修正</x:v>
+        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
       </x:c>
       <x:c r="G12" s="18" t="str">
-        <x:v>夹杂尺寸/密度、钢液物性、流场尺度</x:v>
+        <x:v>案例模板、参数空间、资源配额</x:v>
       </x:c>
       <x:c r="H12" s="18" t="str">
-        <x:v>上浮速度、停留时间、捕获概率</x:v>
+        <x:v>运行状态、结果索引、失败原因</x:v>
       </x:c>
       <x:c r="I12" s="18" t="str">
-        <x:v>显式夹杂尺寸/密度、钢液物性和流动尺度</x:v>
+        <x:v>显式参数空间、案例模板和资源配额</x:v>
       </x:c>
       <x:c r="J12" s="18" t="str">
         <x:v>否</x:v>
@@ -2001,19 +2001,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L12" s="18" t="str">
-        <x:v>Stokes与阻力系数分段关联</x:v>
+        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
       </x:c>
       <x:c r="M12" s="18" t="str">
-        <x:v>C002,C010</x:v>
+        <x:v>G005,G013</x:v>
       </x:c>
       <x:c r="N12" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O12" s="18" t="str">
-        <x:v>不使用质量检测标签</x:v>
+        <x:v>不读取现场数据；只编排批准案例</x:v>
       </x:c>
       <x:c r="P12" s="18" t="str">
-        <x:v>calc_inclusion_float_time</x:v>
+        <x:v>run_parametric_simulation_batch</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" hidden="0" customHeight="1">
@@ -2021,28 +2021,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="D13" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>一维传热PDE求解</x:v>
+        <x:v>插值与查表服务</x:v>
       </x:c>
       <x:c r="F13" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积</x:v>
+        <x:v>多维规则网格/散点插值+缓存</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
-        <x:v>几何、物性、热源、初边值</x:v>
+        <x:v>查询点、表格版本、外推策略</x:v>
       </x:c>
       <x:c r="H13" s="18" t="str">
-        <x:v>温度场、热流、能量闭合</x:v>
+        <x:v>插值值、距离、是否外推</x:v>
       </x:c>
       <x:c r="I13" s="18" t="str">
-        <x:v>显式几何、物性、热源和初边值</x:v>
+        <x:v>调用方上传或选择版本化查找表</x:v>
       </x:c>
       <x:c r="J13" s="18" t="str">
         <x:v>否</x:v>
@@ -2051,19 +2051,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L13" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积与能量闭合</x:v>
+        <x:v>规则网格/散点插值和外推距离</x:v>
       </x:c>
       <x:c r="M13" s="18" t="str">
-        <x:v>G001,G002,T001</x:v>
+        <x:v>A004</x:v>
       </x:c>
       <x:c r="N13" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O13" s="18" t="str">
-        <x:v>纯数值PDE，不使用现场数据</x:v>
+        <x:v>不连接企业实时表</x:v>
       </x:c>
       <x:c r="P13" s="18" t="str">
-        <x:v>solve_heat_pde_1d</x:v>
+        <x:v>interpolate_lookup_table</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" hidden="0" customHeight="1">
@@ -2071,28 +2071,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="C14" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="D14" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>反应ODE求解</x:v>
+        <x:v>敏感性分析</x:v>
       </x:c>
       <x:c r="F14" s="18" t="str">
-        <x:v>刚性/非刚性ODE自适应积分</x:v>
+        <x:v>局部导数、Morris/Sobol可选</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
-        <x:v>反应网络、速率、初值、时间区间</x:v>
+        <x:v>模型、参数范围、采样预算</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
-        <x:v>状态轨迹、事件、收敛信息</x:v>
+        <x:v>敏感度排序、交互效应</x:v>
       </x:c>
       <x:c r="I14" s="18" t="str">
-        <x:v>显式反应网络、速率表达式和初值</x:v>
+        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
       </x:c>
       <x:c r="J14" s="18" t="str">
         <x:v>否</x:v>
@@ -2101,19 +2101,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L14" s="18" t="str">
-        <x:v>自适应刚性/非刚性ODE积分</x:v>
+        <x:v>局部导数、Morris/Sobol</x:v>
       </x:c>
       <x:c r="M14" s="18" t="str">
-        <x:v>C001,G002</x:v>
+        <x:v>A010,G008</x:v>
       </x:c>
       <x:c r="N14" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O14" s="18" t="str">
-        <x:v>纯数值求解，不训练</x:v>
+        <x:v>离线分析，不使用历史成功率</x:v>
       </x:c>
       <x:c r="P14" s="18" t="str">
-        <x:v>solve_reaction_ode</x:v>
+        <x:v>run_sensitivity_analysis</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" hidden="0" customHeight="1">
@@ -2121,28 +2121,28 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>CFD参数化案例生成</x:v>
+        <x:v>Monte Carlo不确定度分析</x:v>
       </x:c>
       <x:c r="F15" s="18" t="str">
-        <x:v>模板渲染+参数/边界条件校验</x:v>
+        <x:v>输入分布采样+模型批量执行</x:v>
       </x:c>
       <x:c r="G15" s="18" t="str">
-        <x:v>几何模板、物性、工况、求解器设置</x:v>
+        <x:v>模型、输入分布、相关性、样本数</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
-        <x:v>可运行CFD案例目录、manifest</x:v>
+        <x:v>输出分布、区间、失效概率</x:v>
       </x:c>
       <x:c r="I15" s="18" t="str">
-        <x:v>调用方显式提交几何模板、物性和工况</x:v>
+        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
       </x:c>
       <x:c r="J15" s="18" t="str">
         <x:v>否</x:v>
@@ -2151,19 +2151,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L15" s="18" t="str">
-        <x:v>OpenFOAM案例模板与schema校验</x:v>
+        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
       </x:c>
       <x:c r="M15" s="18" t="str">
-        <x:v>G001,G002,G013</x:v>
+        <x:v>A010,G006</x:v>
       </x:c>
       <x:c r="N15" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O15" s="18" t="str">
-        <x:v>DS042从必需来源中删除</x:v>
+        <x:v>离线不确定度分析</x:v>
       </x:c>
       <x:c r="P15" s="18" t="str">
-        <x:v>generate_cfd_case</x:v>
+        <x:v>run_monte_carlo_uncertainty</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" hidden="0" customHeight="1">
@@ -2171,28 +2171,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="C16" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="D16" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>参数化仿真批处理</x:v>
+        <x:v>贝叶斯优化</x:v>
       </x:c>
       <x:c r="F16" s="18" t="str">
-        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
+        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
       </x:c>
       <x:c r="G16" s="18" t="str">
-        <x:v>案例模板、参数空间、资源配额</x:v>
+        <x:v>目标函数、约束、变量范围、预算</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
-        <x:v>运行状态、结果索引、失败原因</x:v>
+        <x:v>推荐下一组参数、最优历史、置信度</x:v>
       </x:c>
       <x:c r="I16" s="18" t="str">
-        <x:v>显式参数空间、案例模板和资源配额</x:v>
+        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
       </x:c>
       <x:c r="J16" s="18" t="str">
         <x:v>否</x:v>
@@ -2201,19 +2201,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L16" s="18" t="str">
-        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
+        <x:v>高斯过程/TPE采集函数</x:v>
       </x:c>
       <x:c r="M16" s="18" t="str">
-        <x:v>G005,G013</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N16" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O16" s="18" t="str">
-        <x:v>不读取现场数据；只编排批准案例</x:v>
+        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
       </x:c>
       <x:c r="P16" s="18" t="str">
-        <x:v>run_parametric_simulation_batch</x:v>
+        <x:v>run_bayesian_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" hidden="0" customHeight="1">
@@ -2221,28 +2221,28 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="C17" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="D17" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>插值与查表服务</x:v>
+        <x:v>多目标优化</x:v>
       </x:c>
       <x:c r="F17" s="18" t="str">
-        <x:v>多维规则网格/散点插值+缓存</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="G17" s="18" t="str">
-        <x:v>查询点、表格版本、外推策略</x:v>
+        <x:v>目标、约束、变量、权重偏好</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
-        <x:v>插值值、距离、是否外推</x:v>
+        <x:v>Pareto解集、折中解、约束状态</x:v>
       </x:c>
       <x:c r="I17" s="18" t="str">
-        <x:v>调用方上传或选择版本化查找表</x:v>
+        <x:v>显式目标、约束、变量范围和偏好</x:v>
       </x:c>
       <x:c r="J17" s="18" t="str">
         <x:v>否</x:v>
@@ -2251,19 +2251,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L17" s="18" t="str">
-        <x:v>规则网格/散点插值和外推距离</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="M17" s="18" t="str">
-        <x:v>A004</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N17" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O17" s="18" t="str">
-        <x:v>不连接企业实时表</x:v>
+        <x:v>不读取企业历史数据</x:v>
       </x:c>
       <x:c r="P17" s="18" t="str">
-        <x:v>interpolate_lookup_table</x:v>
+        <x:v>run_multiobjective_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" hidden="0" customHeight="1">
@@ -2271,28 +2271,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="C18" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="D18" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E18" s="18" t="str">
-        <x:v>敏感性分析</x:v>
+        <x:v>约束规则校验器</x:v>
       </x:c>
       <x:c r="F18" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol可选</x:v>
+        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
       </x:c>
       <x:c r="G18" s="18" t="str">
-        <x:v>模型、参数范围、采样预算</x:v>
+        <x:v>模型输入输出、上下文、规则版本</x:v>
       </x:c>
       <x:c r="H18" s="18" t="str">
-        <x:v>敏感度排序、交互效应</x:v>
+        <x:v>通过/失败、违反规则、修复建议</x:v>
       </x:c>
       <x:c r="I18" s="18" t="str">
-        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
+        <x:v>显式模型输入输出与版本化JSON规则</x:v>
       </x:c>
       <x:c r="J18" s="18" t="str">
         <x:v>否</x:v>
@@ -2301,220 +2301,92 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L18" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol</x:v>
+        <x:v>表达式树、物料/能量与工艺边界</x:v>
       </x:c>
       <x:c r="M18" s="18" t="str">
-        <x:v>A010,G008</x:v>
+        <x:v>A005</x:v>
       </x:c>
       <x:c r="N18" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O18" s="18" t="str">
-        <x:v>离线分析，不使用历史成功率</x:v>
+        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
       </x:c>
       <x:c r="P18" s="18" t="str">
-        <x:v>run_sensitivity_analysis</x:v>
+        <x:v>validate_constraints</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" hidden="0" customHeight="1">
-      <x:c r="A19" s="18" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B19" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="C19" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="D19" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E19" s="18" t="str">
-        <x:v>Monte Carlo不确定度分析</x:v>
-      </x:c>
-      <x:c r="F19" s="18" t="str">
-        <x:v>输入分布采样+模型批量执行</x:v>
-      </x:c>
-      <x:c r="G19" s="18" t="str">
-        <x:v>模型、输入分布、相关性、样本数</x:v>
-      </x:c>
-      <x:c r="H19" s="18" t="str">
-        <x:v>输出分布、区间、失效概率</x:v>
-      </x:c>
-      <x:c r="I19" s="18" t="str">
-        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
-      </x:c>
-      <x:c r="J19" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K19" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L19" s="18" t="str">
-        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
-      </x:c>
-      <x:c r="M19" s="18" t="str">
-        <x:v>A010,G006</x:v>
-      </x:c>
-      <x:c r="N19" s="18" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="O19" s="18" t="str">
-        <x:v>离线不确定度分析</x:v>
-      </x:c>
-      <x:c r="P19" s="18" t="str">
-        <x:v>run_monte_carlo_uncertainty</x:v>
-      </x:c>
+      <x:c r="A19" s="18"/>
+      <x:c r="B19" s="18"/>
+      <x:c r="C19" s="18"/>
+      <x:c r="D19" s="18"/>
+      <x:c r="E19" s="18"/>
+      <x:c r="F19" s="18"/>
+      <x:c r="G19" s="18"/>
+      <x:c r="H19" s="18"/>
+      <x:c r="I19" s="18"/>
+      <x:c r="J19" s="18"/>
+      <x:c r="K19" s="18"/>
+      <x:c r="L19" s="18"/>
+      <x:c r="M19" s="18"/>
+      <x:c r="N19" s="18"/>
+      <x:c r="O19" s="18"/>
+      <x:c r="P19" s="18"/>
     </x:row>
     <x:row r="20" ht="42" hidden="0" customHeight="1">
-      <x:c r="A20" s="18" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B20" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="C20" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="D20" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E20" s="18" t="str">
-        <x:v>贝叶斯优化</x:v>
-      </x:c>
-      <x:c r="F20" s="18" t="str">
-        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
-      </x:c>
-      <x:c r="G20" s="18" t="str">
-        <x:v>目标函数、约束、变量范围、预算</x:v>
-      </x:c>
-      <x:c r="H20" s="18" t="str">
-        <x:v>推荐下一组参数、最优历史、置信度</x:v>
-      </x:c>
-      <x:c r="I20" s="18" t="str">
-        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
-      </x:c>
-      <x:c r="J20" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K20" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L20" s="18" t="str">
-        <x:v>高斯过程/TPE采集函数</x:v>
-      </x:c>
-      <x:c r="M20" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N20" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O20" s="18" t="str">
-        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
-      </x:c>
-      <x:c r="P20" s="18" t="str">
-        <x:v>run_bayesian_optimization</x:v>
-      </x:c>
+      <x:c r="A20" s="18"/>
+      <x:c r="B20" s="18"/>
+      <x:c r="C20" s="18"/>
+      <x:c r="D20" s="18"/>
+      <x:c r="E20" s="18"/>
+      <x:c r="F20" s="18"/>
+      <x:c r="G20" s="18"/>
+      <x:c r="H20" s="18"/>
+      <x:c r="I20" s="18"/>
+      <x:c r="J20" s="18"/>
+      <x:c r="K20" s="18"/>
+      <x:c r="L20" s="18"/>
+      <x:c r="M20" s="18"/>
+      <x:c r="N20" s="18"/>
+      <x:c r="O20" s="18"/>
+      <x:c r="P20" s="18"/>
     </x:row>
     <x:row r="21" ht="42" hidden="0" customHeight="1">
-      <x:c r="A21" s="18" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B21" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="C21" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="D21" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E21" s="18" t="str">
-        <x:v>多目标优化</x:v>
-      </x:c>
-      <x:c r="F21" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="G21" s="18" t="str">
-        <x:v>目标、约束、变量、权重偏好</x:v>
-      </x:c>
-      <x:c r="H21" s="18" t="str">
-        <x:v>Pareto解集、折中解、约束状态</x:v>
-      </x:c>
-      <x:c r="I21" s="18" t="str">
-        <x:v>显式目标、约束、变量范围和偏好</x:v>
-      </x:c>
-      <x:c r="J21" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K21" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L21" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="M21" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N21" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O21" s="18" t="str">
-        <x:v>不读取企业历史数据</x:v>
-      </x:c>
-      <x:c r="P21" s="18" t="str">
-        <x:v>run_multiobjective_optimization</x:v>
-      </x:c>
+      <x:c r="A21" s="18"/>
+      <x:c r="B21" s="18"/>
+      <x:c r="C21" s="18"/>
+      <x:c r="D21" s="18"/>
+      <x:c r="E21" s="18"/>
+      <x:c r="F21" s="18"/>
+      <x:c r="G21" s="18"/>
+      <x:c r="H21" s="18"/>
+      <x:c r="I21" s="18"/>
+      <x:c r="J21" s="18"/>
+      <x:c r="K21" s="18"/>
+      <x:c r="L21" s="18"/>
+      <x:c r="M21" s="18"/>
+      <x:c r="N21" s="18"/>
+      <x:c r="O21" s="18"/>
+      <x:c r="P21" s="18"/>
     </x:row>
     <x:row r="22" ht="42" hidden="0" customHeight="1">
-      <x:c r="A22" s="18" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B22" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="C22" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="D22" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E22" s="18" t="str">
-        <x:v>约束规则校验器</x:v>
-      </x:c>
-      <x:c r="F22" s="18" t="str">
-        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="G22" s="18" t="str">
-        <x:v>模型输入输出、上下文、规则版本</x:v>
-      </x:c>
-      <x:c r="H22" s="18" t="str">
-        <x:v>通过/失败、违反规则、修复建议</x:v>
-      </x:c>
-      <x:c r="I22" s="18" t="str">
-        <x:v>显式模型输入输出与版本化JSON规则</x:v>
-      </x:c>
-      <x:c r="J22" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K22" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L22" s="18" t="str">
-        <x:v>表达式树、物料/能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="M22" s="18" t="str">
-        <x:v>A005</x:v>
-      </x:c>
-      <x:c r="N22" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O22" s="18" t="str">
-        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
-      </x:c>
-      <x:c r="P22" s="18" t="str">
-        <x:v>validate_constraints</x:v>
-      </x:c>
+      <x:c r="A22" s="18"/>
+      <x:c r="B22" s="18"/>
+      <x:c r="C22" s="18"/>
+      <x:c r="D22" s="18"/>
+      <x:c r="E22" s="18"/>
+      <x:c r="F22" s="18"/>
+      <x:c r="G22" s="18"/>
+      <x:c r="H22" s="18"/>
+      <x:c r="I22" s="18"/>
+      <x:c r="J22" s="18"/>
+      <x:c r="K22" s="18"/>
+      <x:c r="L22" s="18"/>
+      <x:c r="M22" s="18"/>
+      <x:c r="N22" s="18"/>
+      <x:c r="O22" s="18"/>
+      <x:c r="P22" s="18"/>
     </x:row>
     <x:row r="23" ht="42" hidden="0" customHeight="1">
       <x:c r="A23" s="18"/>
@@ -7150,13 +7022,13 @@
         <x:v>Rist操作线</x:v>
       </x:c>
       <x:c r="D87" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E87" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W14</x:v>
       </x:c>
       <x:c r="F87" s="18" t="str">
-        <x:v>E006</x:v>
+        <x:v>E106</x:v>
       </x:c>
       <x:c r="G87" s="18" t="str">
         <x:v>是</x:v>
@@ -7174,10 +7046,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L87" s="18" t="str">
-        <x:v>planned.e106.v1</x:v>
+        <x:v>metallurgy.catalog.e006.complete_rist_operating_line.v1</x:v>
       </x:c>
       <x:c r="M87" s="18" t="str">
-        <x:v>不修改既有E006；新增完整目录能力</x:v>
+        <x:v>catalog_equivalent_different_runtime_code</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="42" hidden="0" customHeight="1">
@@ -7191,13 +7063,13 @@
         <x:v>喷煤等效替代</x:v>
       </x:c>
       <x:c r="D88" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E88" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W14</x:v>
       </x:c>
       <x:c r="F88" s="18" t="str">
-        <x:v>E009</x:v>
+        <x:v>E109</x:v>
       </x:c>
       <x:c r="G88" s="18" t="str">
         <x:v>是</x:v>
@@ -7215,10 +7087,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L88" s="18" t="str">
-        <x:v>planned.e109.v1</x:v>
+        <x:v>metallurgy.catalog.e009.complete_pci_replacement.v1</x:v>
       </x:c>
       <x:c r="M88" s="18" t="str">
-        <x:v>不修改既有E009范围变体</x:v>
+        <x:v>catalog_equivalent_different_runtime_code</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="42" hidden="0" customHeight="1">
@@ -7232,10 +7104,10 @@
         <x:v>炉顶煤气组成</x:v>
       </x:c>
       <x:c r="D89" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E89" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W14</x:v>
       </x:c>
       <x:c r="F89" s="18" t="str">
         <x:v>E010</x:v>
@@ -7256,10 +7128,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L89" s="18" t="str">
-        <x:v>planned.e010.v1</x:v>
+        <x:v>metallurgy.catalog.e010.bf_top_gas_composition.v1</x:v>
       </x:c>
       <x:c r="M89" s="18" t="str">
-        <x:v>输出理论煤气组成，不接在线分析仪</x:v>
+        <x:v>same</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="42" hidden="0" customHeight="1">
@@ -7273,10 +7145,10 @@
         <x:v>风口回旋区绝热火焰温度</x:v>
       </x:c>
       <x:c r="D90" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E90" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W14</x:v>
       </x:c>
       <x:c r="F90" s="18" t="str">
         <x:v>E013</x:v>
@@ -7297,10 +7169,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L90" s="18" t="str">
-        <x:v>planned.e013.v1</x:v>
+        <x:v>metallurgy.catalog.e013.raceway_adiabatic_flame_temperature.v1</x:v>
       </x:c>
       <x:c r="M90" s="18" t="str">
-        <x:v>作为离线理论RAFT，不依赖风口传感器</x:v>
+        <x:v>same</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="42" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
docs(tools): sync 120-tool catalog to 105 implemented
</commit_message>
<xml_diff>
--- a/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
+++ b/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Re4b119dcd6514a5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R9d1b3c690f7046d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留17" sheetId="3" r:id="Re38b9a8665a549b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="Rbca693d69f854281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="Rbeefa90f772043d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R54e65da23d204b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R778e46c669f44355"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留13" sheetId="3" r:id="R4514ecda2bb845b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="Rdbb5f2b2b9f74002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="Rdff43cb92bb24a60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -280,6 +280,30 @@
 </x:styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RetainedTools13" displayName="RetainedTools13" ref="A1:P14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="16">
+    <x:tableColumn id="1" name="顺序"/>
+    <x:tableColumn id="2" name="运行时ID"/>
+    <x:tableColumn id="3" name="目录ID"/>
+    <x:tableColumn id="4" name="场景"/>
+    <x:tableColumn id="5" name="工具名称"/>
+    <x:tableColumn id="6" name="调整后方法"/>
+    <x:tableColumn id="7" name="主要输入"/>
+    <x:tableColumn id="8" name="主要输出"/>
+    <x:tableColumn id="9" name="调整后数据策略"/>
+    <x:tableColumn id="10" name="现场数据依赖"/>
+    <x:tableColumn id="11" name="训练/权重"/>
+    <x:tableColumn id="12" name="依据"/>
+    <x:tableColumn id="13" name="工具依赖"/>
+    <x:tableColumn id="14" name="难度"/>
+    <x:tableColumn id="15" name="相对原表调整"/>
+    <x:tableColumn id="16" name="API函数名"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -509,7 +533,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>基线：main @ 2028237；P1-W14新增4项后已实现101项，既有97项实现保持原样。</x:v>
+        <x:v>基线：main @ 60a3b67；P1-W15新增E015、E020、F008、F018共4项后已实现105项，既有101项实现保持原样。</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -540,10 +564,10 @@
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:f>COUNTIF('最终120路线'!$D$2:$D$121,"已实现")</x:f>
-        <x:v>101</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>已实现101项不改ID、不撤销资格；P1-W14新增E106、E109、E010、E013共4项。</x:v>
+        <x:v>1. 已实现105项不改ID、不撤销资格；P1-W15新增E015、E020、F008、F018共4项。</x:v>
       </x:c>
       <x:c r="E6" s="27"/>
       <x:c r="F6" s="27"/>
@@ -556,7 +580,7 @@
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:f>COUNTIFS('最终120路线'!$D$2:$D$121,"已实现",'最终120路线'!$G$2:$G$121,"是")</x:f>
-        <x:v>83</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
         <x:v>2. 延期项不注册、不生成空Schema、不计入count_eligible。</x:v>
@@ -572,7 +596,7 @@
       </x:c>
       <x:c r="B8" s="20" t="n">
         <x:f>120-B7</x:f>
-        <x:v>37</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>3. 后续工具不得以DS042、现场时序、企业标签或本地训练权重为准入前提。</x:v>
@@ -603,8 +627,8 @@
         <x:v>后续保留并去现场化</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:f>COUNTA('后续保留17'!$A$2:$A$18)</x:f>
-        <x:v>17</x:v>
+        <x:f>COUNTA('后续保留13'!$A$2:$A$14)</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D10" s="27" t="str">
         <x:v>5. 允许使用公开算法、批准数据库和仓库内版本化常数。</x:v>
@@ -636,7 +660,7 @@
       </x:c>
       <x:c r="B12" s="20" t="n">
         <x:f>B10+B11</x:f>
-        <x:v>19</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
         <x:v>7. 任何未来恢复的现场模型必须另行完成数据授权、脱敏和时序验证。</x:v>
@@ -657,7 +681,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>计数闭合：101 已实现 + 17 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
+        <x:v>计数闭合：105 已实现 + 13 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
       </x:c>
       <x:c r="B15" s="31"/>
       <x:c r="C15" s="31"/>
@@ -1471,28 +1495,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="18" t="str">
-        <x:v>E015</x:v>
+        <x:v>F009</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
-        <x:v>E015</x:v>
+        <x:v>F009</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
-        <x:v>透气性指数</x:v>
+        <x:v>二冷分区水量分配</x:v>
       </x:c>
       <x:c r="F2" s="18" t="str">
-        <x:v>单工况透气性指数；删除趋势异常输出</x:v>
+        <x:v>各区换热模型+温度/回温约束</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
-        <x:v>压差、风量、炉顶压力、料线</x:v>
+        <x:v>总水量、区段、喷嘴、拉速、目标温度</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
-        <x:v>透气性指数、趋势异常</x:v>
+        <x:v>分区水量、温度曲线、约束余量</x:v>
       </x:c>
       <x:c r="I2" s="18" t="str">
-        <x:v>调用方显式提供压差、风量、炉顶压力和料柱高度</x:v>
+        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
         <x:v>否</x:v>
@@ -1501,19 +1525,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L2" s="18" t="str">
-        <x:v>压差—流量归一化指数</x:v>
+        <x:v>分区热平衡与约束优化</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>E014</x:v>
+        <x:v>F005,F008,G012</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O2" s="18" t="str">
-        <x:v>不读取连续时序；不提供炉况预警</x:v>
+        <x:v>作为离线方案，不连接阀门或PLC</x:v>
       </x:c>
       <x:c r="P2" s="18" t="str">
-        <x:v>calc_permeability_index</x:v>
+        <x:v>allocate_secondary_cooling_water</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1521,28 +1545,28 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="18" t="str">
-        <x:v>E020</x:v>
+        <x:v>F011</x:v>
       </x:c>
       <x:c r="C3" s="18" t="str">
-        <x:v>E020</x:v>
+        <x:v>F011</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
-        <x:v>高炉低碳</x:v>
+        <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
-        <x:v>高炉碳足迹</x:v>
+        <x:v>拉速优化</x:v>
       </x:c>
       <x:c r="F3" s="18" t="str">
-        <x:v>活动数据×排放因子；工序边界与分配规则</x:v>
+        <x:v>产量、凝固终点、温度、质量风险多目标优化</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
-        <x:v>焦/煤/电/气/原料/产量、因子版本</x:v>
+        <x:v>钢种、断面、温度、水量、设备约束</x:v>
       </x:c>
       <x:c r="H3" s="18" t="str">
-        <x:v>tCO2e/tHM、分项排放、范围说明</x:v>
+        <x:v>拉速建议、风险/产量权衡</x:v>
       </x:c>
       <x:c r="I3" s="18" t="str">
-        <x:v>调用方显式提供活动数据；排放因子使用公开版本化资产</x:v>
+        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
       </x:c>
       <x:c r="J3" s="18" t="str">
         <x:v>否</x:v>
@@ -1551,19 +1575,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L3" s="18" t="str">
-        <x:v>ISO 14040/14044与GHG Protocol边界记录</x:v>
+        <x:v>F005/F006物理约束下离线搜索</x:v>
       </x:c>
       <x:c r="M3" s="18" t="str">
-        <x:v>E001,E003,E005</x:v>
+        <x:v>F005,F006,F009,G012</x:v>
       </x:c>
       <x:c r="N3" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O3" s="18" t="str">
-        <x:v>不读取企业生产数据库</x:v>
+        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
       </x:c>
       <x:c r="P3" s="18" t="str">
-        <x:v>calc_bf_carbon_footprint</x:v>
+        <x:v>optimize_casting_speed</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" hidden="0" customHeight="1">
@@ -1571,28 +1595,28 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
-        <x:v>F008</x:v>
+        <x:v>F014</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>F008</x:v>
+        <x:v>F014</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>二冷总水量计算</x:v>
+        <x:v>铸坯热应力/应变</x:v>
       </x:c>
       <x:c r="F4" s="18" t="str">
-        <x:v>目标表面温度/比水量经验模型</x:v>
+        <x:v>温度场驱动热弹塑性/裂纹判据</x:v>
       </x:c>
       <x:c r="G4" s="18" t="str">
-        <x:v>钢种、断面、拉速、目标温度</x:v>
+        <x:v>温度场、材料高温力学、边界条件</x:v>
       </x:c>
       <x:c r="H4" s="18" t="str">
-        <x:v>总水量、比水量</x:v>
+        <x:v>应力/应变、危险位置</x:v>
       </x:c>
       <x:c r="I4" s="18" t="str">
-        <x:v>显式断面、拉速、目标热负荷/比水量参数</x:v>
+        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
       </x:c>
       <x:c r="J4" s="18" t="str">
         <x:v>否</x:v>
@@ -1601,19 +1625,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L4" s="18" t="str">
-        <x:v>质量流量与比水量/热量平衡</x:v>
+        <x:v>热应变与简化弹塑性/有限元</x:v>
       </x:c>
       <x:c r="M4" s="18" t="str">
-        <x:v>F003,F005</x:v>
+        <x:v>F005,G003</x:v>
       </x:c>
       <x:c r="N4" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O4" s="18" t="str">
-        <x:v>不从历史浇次拟合参数</x:v>
+        <x:v>不需要现场测温；仅分析显式温度场</x:v>
       </x:c>
       <x:c r="P4" s="18" t="str">
-        <x:v>calc_total_secondary_cooling_water</x:v>
+        <x:v>calc_casting_thermal_stress</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" hidden="0" customHeight="1">
@@ -1621,28 +1645,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G003</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G003</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>二冷分区水量分配</x:v>
+        <x:v>一维传热PDE求解</x:v>
       </x:c>
       <x:c r="F5" s="18" t="str">
-        <x:v>各区换热模型+温度/回温约束</x:v>
+        <x:v>一维导热有限差分/有限体积</x:v>
       </x:c>
       <x:c r="G5" s="18" t="str">
-        <x:v>总水量、区段、喷嘴、拉速、目标温度</x:v>
+        <x:v>几何、物性、热源、初边值</x:v>
       </x:c>
       <x:c r="H5" s="18" t="str">
-        <x:v>分区水量、温度曲线、约束余量</x:v>
+        <x:v>温度场、热流、能量闭合</x:v>
       </x:c>
       <x:c r="I5" s="18" t="str">
-        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
+        <x:v>显式几何、物性、热源和初边值</x:v>
       </x:c>
       <x:c r="J5" s="18" t="str">
         <x:v>否</x:v>
@@ -1651,19 +1675,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L5" s="18" t="str">
-        <x:v>分区热平衡与约束优化</x:v>
+        <x:v>一维导热有限差分/有限体积与能量闭合</x:v>
       </x:c>
       <x:c r="M5" s="18" t="str">
-        <x:v>F005,F008,G012</x:v>
+        <x:v>G001,G002,T001</x:v>
       </x:c>
       <x:c r="N5" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O5" s="18" t="str">
-        <x:v>作为离线方案，不连接阀门或PLC</x:v>
+        <x:v>纯数值PDE，不使用现场数据</x:v>
       </x:c>
       <x:c r="P5" s="18" t="str">
-        <x:v>allocate_secondary_cooling_water</x:v>
+        <x:v>solve_heat_pde_1d</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" hidden="0" customHeight="1">
@@ -1671,28 +1695,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>拉速优化</x:v>
+        <x:v>反应ODE求解</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>产量、凝固终点、温度、质量风险多目标优化</x:v>
+        <x:v>刚性/非刚性ODE自适应积分</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
-        <x:v>钢种、断面、温度、水量、设备约束</x:v>
+        <x:v>反应网络、速率、初值、时间区间</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
-        <x:v>拉速建议、风险/产量权衡</x:v>
+        <x:v>状态轨迹、事件、收敛信息</x:v>
       </x:c>
       <x:c r="I6" s="18" t="str">
-        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
+        <x:v>显式反应网络、速率表达式和初值</x:v>
       </x:c>
       <x:c r="J6" s="18" t="str">
         <x:v>否</x:v>
@@ -1701,19 +1725,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L6" s="18" t="str">
-        <x:v>F005/F006物理约束下离线搜索</x:v>
+        <x:v>自适应刚性/非刚性ODE积分</x:v>
       </x:c>
       <x:c r="M6" s="18" t="str">
-        <x:v>F005,F006,F009,G012</x:v>
+        <x:v>C001,G002</x:v>
       </x:c>
       <x:c r="N6" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O6" s="18" t="str">
-        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
+        <x:v>纯数值求解，不训练</x:v>
       </x:c>
       <x:c r="P6" s="18" t="str">
-        <x:v>optimize_casting_speed</x:v>
+        <x:v>solve_reaction_ode</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" hidden="0" customHeight="1">
@@ -1721,28 +1745,28 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="D7" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>铸坯热应力/应变</x:v>
+        <x:v>CFD参数化案例生成</x:v>
       </x:c>
       <x:c r="F7" s="18" t="str">
-        <x:v>温度场驱动热弹塑性/裂纹判据</x:v>
+        <x:v>模板渲染+参数/边界条件校验</x:v>
       </x:c>
       <x:c r="G7" s="18" t="str">
-        <x:v>温度场、材料高温力学、边界条件</x:v>
+        <x:v>几何模板、物性、工况、求解器设置</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
-        <x:v>应力/应变、危险位置</x:v>
+        <x:v>可运行CFD案例目录、manifest</x:v>
       </x:c>
       <x:c r="I7" s="18" t="str">
-        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
+        <x:v>调用方显式提交几何模板、物性和工况</x:v>
       </x:c>
       <x:c r="J7" s="18" t="str">
         <x:v>否</x:v>
@@ -1751,19 +1775,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L7" s="18" t="str">
-        <x:v>热应变与简化弹塑性/有限元</x:v>
+        <x:v>OpenFOAM案例模板与schema校验</x:v>
       </x:c>
       <x:c r="M7" s="18" t="str">
-        <x:v>F005,G003</x:v>
+        <x:v>G001,G002,G013</x:v>
       </x:c>
       <x:c r="N7" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O7" s="18" t="str">
-        <x:v>不需要现场测温；仅分析显式温度场</x:v>
+        <x:v>DS042从必需来源中删除</x:v>
       </x:c>
       <x:c r="P7" s="18" t="str">
-        <x:v>calc_casting_thermal_stress</x:v>
+        <x:v>generate_cfd_case</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" hidden="0" customHeight="1">
@@ -1771,28 +1795,28 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>F018</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>F018</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>夹杂物上浮时间</x:v>
+        <x:v>参数化仿真批处理</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>Stokes上浮+流场修正</x:v>
+        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
-        <x:v>夹杂尺寸/密度、钢液物性、流场尺度</x:v>
+        <x:v>案例模板、参数空间、资源配额</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
-        <x:v>上浮速度、停留时间、捕获概率</x:v>
+        <x:v>运行状态、结果索引、失败原因</x:v>
       </x:c>
       <x:c r="I8" s="18" t="str">
-        <x:v>显式夹杂尺寸/密度、钢液物性和流动尺度</x:v>
+        <x:v>显式参数空间、案例模板和资源配额</x:v>
       </x:c>
       <x:c r="J8" s="18" t="str">
         <x:v>否</x:v>
@@ -1801,19 +1825,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L8" s="18" t="str">
-        <x:v>Stokes与阻力系数分段关联</x:v>
+        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
       </x:c>
       <x:c r="M8" s="18" t="str">
-        <x:v>C002,C010</x:v>
+        <x:v>G005,G013</x:v>
       </x:c>
       <x:c r="N8" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O8" s="18" t="str">
-        <x:v>不使用质量检测标签</x:v>
+        <x:v>不读取现场数据；只编排批准案例</x:v>
       </x:c>
       <x:c r="P8" s="18" t="str">
-        <x:v>calc_inclusion_float_time</x:v>
+        <x:v>run_parametric_simulation_batch</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" hidden="0" customHeight="1">
@@ -1821,28 +1845,28 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>一维传热PDE求解</x:v>
+        <x:v>插值与查表服务</x:v>
       </x:c>
       <x:c r="F9" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积</x:v>
+        <x:v>多维规则网格/散点插值+缓存</x:v>
       </x:c>
       <x:c r="G9" s="18" t="str">
-        <x:v>几何、物性、热源、初边值</x:v>
+        <x:v>查询点、表格版本、外推策略</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
-        <x:v>温度场、热流、能量闭合</x:v>
+        <x:v>插值值、距离、是否外推</x:v>
       </x:c>
       <x:c r="I9" s="18" t="str">
-        <x:v>显式几何、物性、热源和初边值</x:v>
+        <x:v>调用方上传或选择版本化查找表</x:v>
       </x:c>
       <x:c r="J9" s="18" t="str">
         <x:v>否</x:v>
@@ -1851,19 +1875,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L9" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积与能量闭合</x:v>
+        <x:v>规则网格/散点插值和外推距离</x:v>
       </x:c>
       <x:c r="M9" s="18" t="str">
-        <x:v>G001,G002,T001</x:v>
+        <x:v>A004</x:v>
       </x:c>
       <x:c r="N9" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O9" s="18" t="str">
-        <x:v>纯数值PDE，不使用现场数据</x:v>
+        <x:v>不连接企业实时表</x:v>
       </x:c>
       <x:c r="P9" s="18" t="str">
-        <x:v>solve_heat_pde_1d</x:v>
+        <x:v>interpolate_lookup_table</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" hidden="0" customHeight="1">
@@ -1871,28 +1895,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>反应ODE求解</x:v>
+        <x:v>敏感性分析</x:v>
       </x:c>
       <x:c r="F10" s="18" t="str">
-        <x:v>刚性/非刚性ODE自适应积分</x:v>
+        <x:v>局部导数、Morris/Sobol可选</x:v>
       </x:c>
       <x:c r="G10" s="18" t="str">
-        <x:v>反应网络、速率、初值、时间区间</x:v>
+        <x:v>模型、参数范围、采样预算</x:v>
       </x:c>
       <x:c r="H10" s="18" t="str">
-        <x:v>状态轨迹、事件、收敛信息</x:v>
+        <x:v>敏感度排序、交互效应</x:v>
       </x:c>
       <x:c r="I10" s="18" t="str">
-        <x:v>显式反应网络、速率表达式和初值</x:v>
+        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
       </x:c>
       <x:c r="J10" s="18" t="str">
         <x:v>否</x:v>
@@ -1901,19 +1925,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L10" s="18" t="str">
-        <x:v>自适应刚性/非刚性ODE积分</x:v>
+        <x:v>局部导数、Morris/Sobol</x:v>
       </x:c>
       <x:c r="M10" s="18" t="str">
-        <x:v>C001,G002</x:v>
+        <x:v>A010,G008</x:v>
       </x:c>
       <x:c r="N10" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O10" s="18" t="str">
-        <x:v>纯数值求解，不训练</x:v>
+        <x:v>离线分析，不使用历史成功率</x:v>
       </x:c>
       <x:c r="P10" s="18" t="str">
-        <x:v>solve_reaction_ode</x:v>
+        <x:v>run_sensitivity_analysis</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" hidden="0" customHeight="1">
@@ -1921,28 +1945,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="D11" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>CFD参数化案例生成</x:v>
+        <x:v>Monte Carlo不确定度分析</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
-        <x:v>模板渲染+参数/边界条件校验</x:v>
+        <x:v>输入分布采样+模型批量执行</x:v>
       </x:c>
       <x:c r="G11" s="18" t="str">
-        <x:v>几何模板、物性、工况、求解器设置</x:v>
+        <x:v>模型、输入分布、相关性、样本数</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
-        <x:v>可运行CFD案例目录、manifest</x:v>
+        <x:v>输出分布、区间、失效概率</x:v>
       </x:c>
       <x:c r="I11" s="18" t="str">
-        <x:v>调用方显式提交几何模板、物性和工况</x:v>
+        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
       </x:c>
       <x:c r="J11" s="18" t="str">
         <x:v>否</x:v>
@@ -1951,19 +1975,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L11" s="18" t="str">
-        <x:v>OpenFOAM案例模板与schema校验</x:v>
+        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
       </x:c>
       <x:c r="M11" s="18" t="str">
-        <x:v>G001,G002,G013</x:v>
+        <x:v>A010,G006</x:v>
       </x:c>
       <x:c r="N11" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O11" s="18" t="str">
-        <x:v>DS042从必需来源中删除</x:v>
+        <x:v>离线不确定度分析</x:v>
       </x:c>
       <x:c r="P11" s="18" t="str">
-        <x:v>generate_cfd_case</x:v>
+        <x:v>run_monte_carlo_uncertainty</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" hidden="0" customHeight="1">
@@ -1971,28 +1995,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="D12" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>参数化仿真批处理</x:v>
+        <x:v>贝叶斯优化</x:v>
       </x:c>
       <x:c r="F12" s="18" t="str">
-        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
+        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
       </x:c>
       <x:c r="G12" s="18" t="str">
-        <x:v>案例模板、参数空间、资源配额</x:v>
+        <x:v>目标函数、约束、变量范围、预算</x:v>
       </x:c>
       <x:c r="H12" s="18" t="str">
-        <x:v>运行状态、结果索引、失败原因</x:v>
+        <x:v>推荐下一组参数、最优历史、置信度</x:v>
       </x:c>
       <x:c r="I12" s="18" t="str">
-        <x:v>显式参数空间、案例模板和资源配额</x:v>
+        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
       </x:c>
       <x:c r="J12" s="18" t="str">
         <x:v>否</x:v>
@@ -2001,19 +2025,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L12" s="18" t="str">
-        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
+        <x:v>高斯过程/TPE采集函数</x:v>
       </x:c>
       <x:c r="M12" s="18" t="str">
-        <x:v>G005,G013</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N12" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O12" s="18" t="str">
-        <x:v>不读取现场数据；只编排批准案例</x:v>
+        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
       </x:c>
       <x:c r="P12" s="18" t="str">
-        <x:v>run_parametric_simulation_batch</x:v>
+        <x:v>run_bayesian_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" hidden="0" customHeight="1">
@@ -2021,28 +2045,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="D13" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>插值与查表服务</x:v>
+        <x:v>多目标优化</x:v>
       </x:c>
       <x:c r="F13" s="18" t="str">
-        <x:v>多维规则网格/散点插值+缓存</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
-        <x:v>查询点、表格版本、外推策略</x:v>
+        <x:v>目标、约束、变量、权重偏好</x:v>
       </x:c>
       <x:c r="H13" s="18" t="str">
-        <x:v>插值值、距离、是否外推</x:v>
+        <x:v>Pareto解集、折中解、约束状态</x:v>
       </x:c>
       <x:c r="I13" s="18" t="str">
-        <x:v>调用方上传或选择版本化查找表</x:v>
+        <x:v>显式目标、约束、变量范围和偏好</x:v>
       </x:c>
       <x:c r="J13" s="18" t="str">
         <x:v>否</x:v>
@@ -2051,19 +2075,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L13" s="18" t="str">
-        <x:v>规则网格/散点插值和外推距离</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="M13" s="18" t="str">
-        <x:v>A004</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N13" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O13" s="18" t="str">
-        <x:v>不连接企业实时表</x:v>
+        <x:v>不读取企业历史数据</x:v>
       </x:c>
       <x:c r="P13" s="18" t="str">
-        <x:v>interpolate_lookup_table</x:v>
+        <x:v>run_multiobjective_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" hidden="0" customHeight="1">
@@ -2071,28 +2095,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="C14" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="D14" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>敏感性分析</x:v>
+        <x:v>约束规则校验器</x:v>
       </x:c>
       <x:c r="F14" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol可选</x:v>
+        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
-        <x:v>模型、参数范围、采样预算</x:v>
+        <x:v>模型输入输出、上下文、规则版本</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
-        <x:v>敏感度排序、交互效应</x:v>
+        <x:v>通过/失败、违反规则、修复建议</x:v>
       </x:c>
       <x:c r="I14" s="18" t="str">
-        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
+        <x:v>显式模型输入输出与版本化JSON规则</x:v>
       </x:c>
       <x:c r="J14" s="18" t="str">
         <x:v>否</x:v>
@@ -2101,220 +2125,92 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L14" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol</x:v>
+        <x:v>表达式树、物料/能量与工艺边界</x:v>
       </x:c>
       <x:c r="M14" s="18" t="str">
-        <x:v>A010,G008</x:v>
+        <x:v>A005</x:v>
       </x:c>
       <x:c r="N14" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O14" s="18" t="str">
-        <x:v>离线分析，不使用历史成功率</x:v>
+        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
       </x:c>
       <x:c r="P14" s="18" t="str">
-        <x:v>run_sensitivity_analysis</x:v>
+        <x:v>validate_constraints</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" hidden="0" customHeight="1">
-      <x:c r="A15" s="18" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B15" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="C15" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="D15" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E15" s="18" t="str">
-        <x:v>Monte Carlo不确定度分析</x:v>
-      </x:c>
-      <x:c r="F15" s="18" t="str">
-        <x:v>输入分布采样+模型批量执行</x:v>
-      </x:c>
-      <x:c r="G15" s="18" t="str">
-        <x:v>模型、输入分布、相关性、样本数</x:v>
-      </x:c>
-      <x:c r="H15" s="18" t="str">
-        <x:v>输出分布、区间、失效概率</x:v>
-      </x:c>
-      <x:c r="I15" s="18" t="str">
-        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
-      </x:c>
-      <x:c r="J15" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K15" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L15" s="18" t="str">
-        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
-      </x:c>
-      <x:c r="M15" s="18" t="str">
-        <x:v>A010,G006</x:v>
-      </x:c>
-      <x:c r="N15" s="18" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="O15" s="18" t="str">
-        <x:v>离线不确定度分析</x:v>
-      </x:c>
-      <x:c r="P15" s="18" t="str">
-        <x:v>run_monte_carlo_uncertainty</x:v>
-      </x:c>
+      <x:c r="A15" s="18"/>
+      <x:c r="B15" s="18"/>
+      <x:c r="C15" s="18"/>
+      <x:c r="D15" s="18"/>
+      <x:c r="E15" s="18"/>
+      <x:c r="F15" s="18"/>
+      <x:c r="G15" s="18"/>
+      <x:c r="H15" s="18"/>
+      <x:c r="I15" s="18"/>
+      <x:c r="J15" s="18"/>
+      <x:c r="K15" s="18"/>
+      <x:c r="L15" s="18"/>
+      <x:c r="M15" s="18"/>
+      <x:c r="N15" s="18"/>
+      <x:c r="O15" s="18"/>
+      <x:c r="P15" s="18"/>
     </x:row>
     <x:row r="16" ht="42" hidden="0" customHeight="1">
-      <x:c r="A16" s="18" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B16" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="C16" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="D16" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E16" s="18" t="str">
-        <x:v>贝叶斯优化</x:v>
-      </x:c>
-      <x:c r="F16" s="18" t="str">
-        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
-      </x:c>
-      <x:c r="G16" s="18" t="str">
-        <x:v>目标函数、约束、变量范围、预算</x:v>
-      </x:c>
-      <x:c r="H16" s="18" t="str">
-        <x:v>推荐下一组参数、最优历史、置信度</x:v>
-      </x:c>
-      <x:c r="I16" s="18" t="str">
-        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
-      </x:c>
-      <x:c r="J16" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K16" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L16" s="18" t="str">
-        <x:v>高斯过程/TPE采集函数</x:v>
-      </x:c>
-      <x:c r="M16" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N16" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O16" s="18" t="str">
-        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
-      </x:c>
-      <x:c r="P16" s="18" t="str">
-        <x:v>run_bayesian_optimization</x:v>
-      </x:c>
+      <x:c r="A16" s="18"/>
+      <x:c r="B16" s="18"/>
+      <x:c r="C16" s="18"/>
+      <x:c r="D16" s="18"/>
+      <x:c r="E16" s="18"/>
+      <x:c r="F16" s="18"/>
+      <x:c r="G16" s="18"/>
+      <x:c r="H16" s="18"/>
+      <x:c r="I16" s="18"/>
+      <x:c r="J16" s="18"/>
+      <x:c r="K16" s="18"/>
+      <x:c r="L16" s="18"/>
+      <x:c r="M16" s="18"/>
+      <x:c r="N16" s="18"/>
+      <x:c r="O16" s="18"/>
+      <x:c r="P16" s="18"/>
     </x:row>
     <x:row r="17" ht="42" hidden="0" customHeight="1">
-      <x:c r="A17" s="18" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B17" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="C17" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="D17" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E17" s="18" t="str">
-        <x:v>多目标优化</x:v>
-      </x:c>
-      <x:c r="F17" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="G17" s="18" t="str">
-        <x:v>目标、约束、变量、权重偏好</x:v>
-      </x:c>
-      <x:c r="H17" s="18" t="str">
-        <x:v>Pareto解集、折中解、约束状态</x:v>
-      </x:c>
-      <x:c r="I17" s="18" t="str">
-        <x:v>显式目标、约束、变量范围和偏好</x:v>
-      </x:c>
-      <x:c r="J17" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K17" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L17" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="M17" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N17" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O17" s="18" t="str">
-        <x:v>不读取企业历史数据</x:v>
-      </x:c>
-      <x:c r="P17" s="18" t="str">
-        <x:v>run_multiobjective_optimization</x:v>
-      </x:c>
+      <x:c r="A17" s="18"/>
+      <x:c r="B17" s="18"/>
+      <x:c r="C17" s="18"/>
+      <x:c r="D17" s="18"/>
+      <x:c r="E17" s="18"/>
+      <x:c r="F17" s="18"/>
+      <x:c r="G17" s="18"/>
+      <x:c r="H17" s="18"/>
+      <x:c r="I17" s="18"/>
+      <x:c r="J17" s="18"/>
+      <x:c r="K17" s="18"/>
+      <x:c r="L17" s="18"/>
+      <x:c r="M17" s="18"/>
+      <x:c r="N17" s="18"/>
+      <x:c r="O17" s="18"/>
+      <x:c r="P17" s="18"/>
     </x:row>
     <x:row r="18" ht="42" hidden="0" customHeight="1">
-      <x:c r="A18" s="18" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B18" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="C18" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="D18" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E18" s="18" t="str">
-        <x:v>约束规则校验器</x:v>
-      </x:c>
-      <x:c r="F18" s="18" t="str">
-        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="G18" s="18" t="str">
-        <x:v>模型输入输出、上下文、规则版本</x:v>
-      </x:c>
-      <x:c r="H18" s="18" t="str">
-        <x:v>通过/失败、违反规则、修复建议</x:v>
-      </x:c>
-      <x:c r="I18" s="18" t="str">
-        <x:v>显式模型输入输出与版本化JSON规则</x:v>
-      </x:c>
-      <x:c r="J18" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K18" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L18" s="18" t="str">
-        <x:v>表达式树、物料/能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="M18" s="18" t="str">
-        <x:v>A005</x:v>
-      </x:c>
-      <x:c r="N18" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O18" s="18" t="str">
-        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
-      </x:c>
-      <x:c r="P18" s="18" t="str">
-        <x:v>validate_constraints</x:v>
-      </x:c>
+      <x:c r="A18" s="18"/>
+      <x:c r="B18" s="18"/>
+      <x:c r="C18" s="18"/>
+      <x:c r="D18" s="18"/>
+      <x:c r="E18" s="18"/>
+      <x:c r="F18" s="18"/>
+      <x:c r="G18" s="18"/>
+      <x:c r="H18" s="18"/>
+      <x:c r="I18" s="18"/>
+      <x:c r="J18" s="18"/>
+      <x:c r="K18" s="18"/>
+      <x:c r="L18" s="18"/>
+      <x:c r="M18" s="18"/>
+      <x:c r="N18" s="18"/>
+      <x:c r="O18" s="18"/>
+      <x:c r="P18" s="18"/>
     </x:row>
     <x:row r="19" ht="42" hidden="0" customHeight="1">
       <x:c r="A19" s="18"/>
@@ -2591,6 +2487,9 @@
     <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="否"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R074b8d7d6b834e89"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -7186,10 +7085,10 @@
         <x:v>透气性指数</x:v>
       </x:c>
       <x:c r="D91" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E91" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W15</x:v>
       </x:c>
       <x:c r="F91" s="18" t="str">
         <x:v>E015</x:v>
@@ -7201,7 +7100,7 @@
         <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="I91" s="18" t="str">
-        <x:v>调用方显式提供压差、风量、炉顶压力和料柱高度</x:v>
+        <x:v>调用方显式提供单工况绝压、标况风量、平均物性、截面积和料柱高度</x:v>
       </x:c>
       <x:c r="J91" s="18" t="str">
         <x:v>否</x:v>
@@ -7210,10 +7109,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L91" s="18" t="str">
-        <x:v>planned.e015.v1</x:v>
+        <x:v>metallurgy.catalog.e015.bf_permeability_resistance_index.v1</x:v>
       </x:c>
       <x:c r="M91" s="18" t="str">
-        <x:v>不读取连续时序；不提供炉况预警</x:v>
+        <x:v>单快照归一化阻力；不读取连续时序、不提供炉况预警</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="42" hidden="0" customHeight="1">
@@ -7227,10 +7126,10 @@
         <x:v>高炉碳足迹</x:v>
       </x:c>
       <x:c r="D92" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E92" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W15</x:v>
       </x:c>
       <x:c r="F92" s="18" t="str">
         <x:v>E020</x:v>
@@ -7242,7 +7141,7 @@
         <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="I92" s="18" t="str">
-        <x:v>调用方显式提供活动数据；排放因子使用公开版本化资产</x:v>
+        <x:v>显式活动数据；PostgreSQL只读查询公开版本化IPCC/MEE因子</x:v>
       </x:c>
       <x:c r="J92" s="18" t="str">
         <x:v>否</x:v>
@@ -7251,10 +7150,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L92" s="18" t="str">
-        <x:v>planned.e020.v1</x:v>
+        <x:v>metallurgy.catalog.e020.bf_carbon_footprint.v1</x:v>
       </x:c>
       <x:c r="M92" s="18" t="str">
-        <x:v>不读取企业生产数据库</x:v>
+        <x:v>透明活动因子账本；不读取企业生产数据库，不替代认证LCA</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="42" hidden="0" customHeight="1">
@@ -7268,10 +7167,10 @@
         <x:v>二冷总水量计算</x:v>
       </x:c>
       <x:c r="D93" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E93" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W15</x:v>
       </x:c>
       <x:c r="F93" s="18" t="str">
         <x:v>F008</x:v>
@@ -7283,7 +7182,7 @@
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="I93" s="18" t="str">
-        <x:v>显式断面、拉速、目标热负荷/比水量参数</x:v>
+        <x:v>显式断面、拉速、钢密度和目标热负荷/比水量参数</x:v>
       </x:c>
       <x:c r="J93" s="18" t="str">
         <x:v>否</x:v>
@@ -7292,10 +7191,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L93" s="18" t="str">
-        <x:v>planned.f008.v1</x:v>
+        <x:v>metallurgy.catalog.f008.total_secondary_cooling_water.v1</x:v>
       </x:c>
       <x:c r="M93" s="18" t="str">
-        <x:v>不从历史浇次拟合参数</x:v>
+        <x:v>稳态总量级；不从历史浇次拟合参数、不分区配水</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="42" hidden="0" customHeight="1">
@@ -7432,10 +7331,10 @@
         <x:v>夹杂物上浮时间</x:v>
       </x:c>
       <x:c r="D97" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E97" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W15</x:v>
       </x:c>
       <x:c r="F97" s="18" t="str">
         <x:v>F018</x:v>
@@ -7447,7 +7346,7 @@
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="I97" s="18" t="str">
-        <x:v>显式夹杂尺寸/密度、钢液物性和流动尺度</x:v>
+        <x:v>显式球形夹杂尺寸/密度、钢液密度/黏度、距离和均匀竖直速度</x:v>
       </x:c>
       <x:c r="J97" s="18" t="str">
         <x:v>否</x:v>
@@ -7456,10 +7355,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L97" s="18" t="str">
-        <x:v>planned.f018.v1</x:v>
+        <x:v>metallurgy.catalog.f018.inclusion_float_time.v1</x:v>
       </x:c>
       <x:c r="M97" s="18" t="str">
-        <x:v>不使用质量检测标签</x:v>
+        <x:v>Stokes/Schiller–Naumann运动学；不使用质量检测标签、不声称捕获概率</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="42" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
docs(tools): sync 120-tool catalog to 109 implemented
</commit_message>
<xml_diff>
--- a/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
+++ b/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R54e65da23d204b20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R778e46c669f44355"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留13" sheetId="3" r:id="R4514ecda2bb845b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="Rdbb5f2b2b9f74002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="Rdff43cb92bb24a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rea36d924c4df4fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R52046e73d1814c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留9" sheetId="3" r:id="R40fc0ca356914585"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R0ee28584436743f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R51e60a944a214602"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -533,7 +533,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>基线：main @ 60a3b67；P1-W15新增E015、E020、F008、F018共4项后已实现105项，既有101项实现保持原样。</x:v>
+        <x:v>基线：main @ b861071；P1-W16新增F009、F011、F014、G003共4项后已实现109项，既有105项实现保持原样。</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -564,10 +564,10 @@
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:f>COUNTIF('最终120路线'!$D$2:$D$121,"已实现")</x:f>
-        <x:v>105</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>1. 已实现105项不改ID、不撤销资格；P1-W15新增E015、E020、F008、F018共4项。</x:v>
+        <x:v>1. 已实现109项不改ID、不撤销资格；P1-W16新增F009、F011、F014、G003共4项。</x:v>
       </x:c>
       <x:c r="E6" s="27"/>
       <x:c r="F6" s="27"/>
@@ -580,7 +580,7 @@
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:f>COUNTIFS('最终120路线'!$D$2:$D$121,"已实现",'最终120路线'!$G$2:$G$121,"是")</x:f>
-        <x:v>87</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
         <x:v>2. 延期项不注册、不生成空Schema、不计入count_eligible。</x:v>
@@ -596,7 +596,7 @@
       </x:c>
       <x:c r="B8" s="20" t="n">
         <x:f>120-B7</x:f>
-        <x:v>33</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>3. 后续工具不得以DS042、现场时序、企业标签或本地训练权重为准入前提。</x:v>
@@ -627,8 +627,8 @@
         <x:v>后续保留并去现场化</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:f>COUNTA('后续保留13'!$A$2:$A$14)</x:f>
-        <x:v>13</x:v>
+        <x:f>COUNTA('后续保留9'!$A$2:$A$10)</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D10" s="27" t="str">
         <x:v>5. 允许使用公开算法、批准数据库和仓库内版本化常数。</x:v>
@@ -660,7 +660,7 @@
       </x:c>
       <x:c r="B12" s="20" t="n">
         <x:f>B10+B11</x:f>
-        <x:v>15</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
         <x:v>7. 任何未来恢复的现场模型必须另行完成数据授权、脱敏和时序验证。</x:v>
@@ -681,7 +681,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>计数闭合：105 已实现 + 13 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
+        <x:v>计数闭合：109 已实现 + 9 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
       </x:c>
       <x:c r="B15" s="31"/>
       <x:c r="C15" s="31"/>
@@ -1495,28 +1495,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
-        <x:v>F009</x:v>
+        <x:v>G004</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
-        <x:v>二冷分区水量分配</x:v>
+        <x:v>反应ODE求解</x:v>
       </x:c>
       <x:c r="F2" s="18" t="str">
-        <x:v>各区换热模型+温度/回温约束</x:v>
+        <x:v>刚性/非刚性ODE自适应积分</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
-        <x:v>总水量、区段、喷嘴、拉速、目标温度</x:v>
+        <x:v>反应网络、速率、初值、时间区间</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
-        <x:v>分区水量、温度曲线、约束余量</x:v>
+        <x:v>状态轨迹、事件、收敛信息</x:v>
       </x:c>
       <x:c r="I2" s="18" t="str">
-        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
+        <x:v>显式反应网络、速率表达式和初值</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
         <x:v>否</x:v>
@@ -1525,19 +1525,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L2" s="18" t="str">
-        <x:v>分区热平衡与约束优化</x:v>
+        <x:v>自适应刚性/非刚性ODE积分</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>F005,F008,G012</x:v>
+        <x:v>C001,G002</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="O2" s="18" t="str">
-        <x:v>作为离线方案，不连接阀门或PLC</x:v>
+        <x:v>纯数值求解，不训练</x:v>
       </x:c>
       <x:c r="P2" s="18" t="str">
-        <x:v>allocate_secondary_cooling_water</x:v>
+        <x:v>solve_reaction_ode</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1545,28 +1545,28 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="C3" s="18" t="str">
-        <x:v>F011</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
-        <x:v>拉速优化</x:v>
+        <x:v>CFD参数化案例生成</x:v>
       </x:c>
       <x:c r="F3" s="18" t="str">
-        <x:v>产量、凝固终点、温度、质量风险多目标优化</x:v>
+        <x:v>模板渲染+参数/边界条件校验</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
-        <x:v>钢种、断面、温度、水量、设备约束</x:v>
+        <x:v>几何模板、物性、工况、求解器设置</x:v>
       </x:c>
       <x:c r="H3" s="18" t="str">
-        <x:v>拉速建议、风险/产量权衡</x:v>
+        <x:v>可运行CFD案例目录、manifest</x:v>
       </x:c>
       <x:c r="I3" s="18" t="str">
-        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
+        <x:v>调用方显式提交几何模板、物性和工况</x:v>
       </x:c>
       <x:c r="J3" s="18" t="str">
         <x:v>否</x:v>
@@ -1575,19 +1575,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L3" s="18" t="str">
-        <x:v>F005/F006物理约束下离线搜索</x:v>
+        <x:v>OpenFOAM案例模板与schema校验</x:v>
       </x:c>
       <x:c r="M3" s="18" t="str">
-        <x:v>F005,F006,F009,G012</x:v>
+        <x:v>G001,G002,G013</x:v>
       </x:c>
       <x:c r="N3" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O3" s="18" t="str">
-        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
+        <x:v>DS042从必需来源中删除</x:v>
       </x:c>
       <x:c r="P3" s="18" t="str">
-        <x:v>optimize_casting_speed</x:v>
+        <x:v>generate_cfd_case</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" hidden="0" customHeight="1">
@@ -1595,28 +1595,28 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>F014</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
-        <x:v>连铸质量与二冷</x:v>
+        <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>铸坯热应力/应变</x:v>
+        <x:v>参数化仿真批处理</x:v>
       </x:c>
       <x:c r="F4" s="18" t="str">
-        <x:v>温度场驱动热弹塑性/裂纹判据</x:v>
+        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
       </x:c>
       <x:c r="G4" s="18" t="str">
-        <x:v>温度场、材料高温力学、边界条件</x:v>
+        <x:v>案例模板、参数空间、资源配额</x:v>
       </x:c>
       <x:c r="H4" s="18" t="str">
-        <x:v>应力/应变、危险位置</x:v>
+        <x:v>运行状态、结果索引、失败原因</x:v>
       </x:c>
       <x:c r="I4" s="18" t="str">
-        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
+        <x:v>显式参数空间、案例模板和资源配额</x:v>
       </x:c>
       <x:c r="J4" s="18" t="str">
         <x:v>否</x:v>
@@ -1625,19 +1625,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L4" s="18" t="str">
-        <x:v>热应变与简化弹塑性/有限元</x:v>
+        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
       </x:c>
       <x:c r="M4" s="18" t="str">
-        <x:v>F005,G003</x:v>
+        <x:v>G005,G013</x:v>
       </x:c>
       <x:c r="N4" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O4" s="18" t="str">
-        <x:v>不需要现场测温；仅分析显式温度场</x:v>
+        <x:v>不读取现场数据；只编排批准案例</x:v>
       </x:c>
       <x:c r="P4" s="18" t="str">
-        <x:v>calc_casting_thermal_stress</x:v>
+        <x:v>run_parametric_simulation_batch</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" hidden="0" customHeight="1">
@@ -1645,28 +1645,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>G003</x:v>
+        <x:v>G008</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>一维传热PDE求解</x:v>
+        <x:v>插值与查表服务</x:v>
       </x:c>
       <x:c r="F5" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积</x:v>
+        <x:v>多维规则网格/散点插值+缓存</x:v>
       </x:c>
       <x:c r="G5" s="18" t="str">
-        <x:v>几何、物性、热源、初边值</x:v>
+        <x:v>查询点、表格版本、外推策略</x:v>
       </x:c>
       <x:c r="H5" s="18" t="str">
-        <x:v>温度场、热流、能量闭合</x:v>
+        <x:v>插值值、距离、是否外推</x:v>
       </x:c>
       <x:c r="I5" s="18" t="str">
-        <x:v>显式几何、物性、热源和初边值</x:v>
+        <x:v>调用方上传或选择版本化查找表</x:v>
       </x:c>
       <x:c r="J5" s="18" t="str">
         <x:v>否</x:v>
@@ -1675,19 +1675,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L5" s="18" t="str">
-        <x:v>一维导热有限差分/有限体积与能量闭合</x:v>
+        <x:v>规则网格/散点插值和外推距离</x:v>
       </x:c>
       <x:c r="M5" s="18" t="str">
-        <x:v>G001,G002,T001</x:v>
+        <x:v>A004</x:v>
       </x:c>
       <x:c r="N5" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O5" s="18" t="str">
-        <x:v>纯数值PDE，不使用现场数据</x:v>
+        <x:v>不连接企业实时表</x:v>
       </x:c>
       <x:c r="P5" s="18" t="str">
-        <x:v>solve_heat_pde_1d</x:v>
+        <x:v>interpolate_lookup_table</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" hidden="0" customHeight="1">
@@ -1695,28 +1695,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G009</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>反应ODE求解</x:v>
+        <x:v>敏感性分析</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>刚性/非刚性ODE自适应积分</x:v>
+        <x:v>局部导数、Morris/Sobol可选</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
-        <x:v>反应网络、速率、初值、时间区间</x:v>
+        <x:v>模型、参数范围、采样预算</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
-        <x:v>状态轨迹、事件、收敛信息</x:v>
+        <x:v>敏感度排序、交互效应</x:v>
       </x:c>
       <x:c r="I6" s="18" t="str">
-        <x:v>显式反应网络、速率表达式和初值</x:v>
+        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
       </x:c>
       <x:c r="J6" s="18" t="str">
         <x:v>否</x:v>
@@ -1725,19 +1725,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L6" s="18" t="str">
-        <x:v>自适应刚性/非刚性ODE积分</x:v>
+        <x:v>局部导数、Morris/Sobol</x:v>
       </x:c>
       <x:c r="M6" s="18" t="str">
-        <x:v>C001,G002</x:v>
+        <x:v>A010,G008</x:v>
       </x:c>
       <x:c r="N6" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O6" s="18" t="str">
-        <x:v>纯数值求解，不训练</x:v>
+        <x:v>离线分析，不使用历史成功率</x:v>
       </x:c>
       <x:c r="P6" s="18" t="str">
-        <x:v>solve_reaction_ode</x:v>
+        <x:v>run_sensitivity_analysis</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" hidden="0" customHeight="1">
@@ -1745,28 +1745,28 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G010</x:v>
       </x:c>
       <x:c r="D7" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>CFD参数化案例生成</x:v>
+        <x:v>Monte Carlo不确定度分析</x:v>
       </x:c>
       <x:c r="F7" s="18" t="str">
-        <x:v>模板渲染+参数/边界条件校验</x:v>
+        <x:v>输入分布采样+模型批量执行</x:v>
       </x:c>
       <x:c r="G7" s="18" t="str">
-        <x:v>几何模板、物性、工况、求解器设置</x:v>
+        <x:v>模型、输入分布、相关性、样本数</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
-        <x:v>可运行CFD案例目录、manifest</x:v>
+        <x:v>输出分布、区间、失效概率</x:v>
       </x:c>
       <x:c r="I7" s="18" t="str">
-        <x:v>调用方显式提交几何模板、物性和工况</x:v>
+        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
       </x:c>
       <x:c r="J7" s="18" t="str">
         <x:v>否</x:v>
@@ -1775,19 +1775,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L7" s="18" t="str">
-        <x:v>OpenFOAM案例模板与schema校验</x:v>
+        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
       </x:c>
       <x:c r="M7" s="18" t="str">
-        <x:v>G001,G002,G013</x:v>
+        <x:v>A010,G006</x:v>
       </x:c>
       <x:c r="N7" s="18" t="str">
-        <x:v>高</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="O7" s="18" t="str">
-        <x:v>DS042从必需来源中删除</x:v>
+        <x:v>离线不确定度分析</x:v>
       </x:c>
       <x:c r="P7" s="18" t="str">
-        <x:v>generate_cfd_case</x:v>
+        <x:v>run_monte_carlo_uncertainty</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" hidden="0" customHeight="1">
@@ -1795,28 +1795,28 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>参数化仿真批处理</x:v>
+        <x:v>贝叶斯优化</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
+        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
-        <x:v>案例模板、参数空间、资源配额</x:v>
+        <x:v>目标函数、约束、变量范围、预算</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
-        <x:v>运行状态、结果索引、失败原因</x:v>
+        <x:v>推荐下一组参数、最优历史、置信度</x:v>
       </x:c>
       <x:c r="I8" s="18" t="str">
-        <x:v>显式参数空间、案例模板和资源配额</x:v>
+        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
       </x:c>
       <x:c r="J8" s="18" t="str">
         <x:v>否</x:v>
@@ -1825,19 +1825,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L8" s="18" t="str">
-        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
+        <x:v>高斯过程/TPE采集函数</x:v>
       </x:c>
       <x:c r="M8" s="18" t="str">
-        <x:v>G005,G013</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N8" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O8" s="18" t="str">
-        <x:v>不读取现场数据；只编排批准案例</x:v>
+        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
       </x:c>
       <x:c r="P8" s="18" t="str">
-        <x:v>run_parametric_simulation_batch</x:v>
+        <x:v>run_bayesian_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" hidden="0" customHeight="1">
@@ -1845,28 +1845,28 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>插值与查表服务</x:v>
+        <x:v>多目标优化</x:v>
       </x:c>
       <x:c r="F9" s="18" t="str">
-        <x:v>多维规则网格/散点插值+缓存</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="G9" s="18" t="str">
-        <x:v>查询点、表格版本、外推策略</x:v>
+        <x:v>目标、约束、变量、权重偏好</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
-        <x:v>插值值、距离、是否外推</x:v>
+        <x:v>Pareto解集、折中解、约束状态</x:v>
       </x:c>
       <x:c r="I9" s="18" t="str">
-        <x:v>调用方上传或选择版本化查找表</x:v>
+        <x:v>显式目标、约束、变量范围和偏好</x:v>
       </x:c>
       <x:c r="J9" s="18" t="str">
         <x:v>否</x:v>
@@ -1875,19 +1875,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L9" s="18" t="str">
-        <x:v>规则网格/散点插值和外推距离</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="M9" s="18" t="str">
-        <x:v>A004</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N9" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O9" s="18" t="str">
-        <x:v>不连接企业实时表</x:v>
+        <x:v>不读取企业历史数据</x:v>
       </x:c>
       <x:c r="P9" s="18" t="str">
-        <x:v>interpolate_lookup_table</x:v>
+        <x:v>run_multiobjective_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" hidden="0" customHeight="1">
@@ -1895,28 +1895,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>敏感性分析</x:v>
+        <x:v>约束规则校验器</x:v>
       </x:c>
       <x:c r="F10" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol可选</x:v>
+        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
       </x:c>
       <x:c r="G10" s="18" t="str">
-        <x:v>模型、参数范围、采样预算</x:v>
+        <x:v>模型输入输出、上下文、规则版本</x:v>
       </x:c>
       <x:c r="H10" s="18" t="str">
-        <x:v>敏感度排序、交互效应</x:v>
+        <x:v>通过/失败、违反规则、修复建议</x:v>
       </x:c>
       <x:c r="I10" s="18" t="str">
-        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
+        <x:v>显式模型输入输出与版本化JSON规则</x:v>
       </x:c>
       <x:c r="J10" s="18" t="str">
         <x:v>否</x:v>
@@ -1925,220 +1925,92 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L10" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol</x:v>
+        <x:v>表达式树、物料/能量与工艺边界</x:v>
       </x:c>
       <x:c r="M10" s="18" t="str">
-        <x:v>A010,G008</x:v>
+        <x:v>A005</x:v>
       </x:c>
       <x:c r="N10" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O10" s="18" t="str">
-        <x:v>离线分析，不使用历史成功率</x:v>
+        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
       </x:c>
       <x:c r="P10" s="18" t="str">
-        <x:v>run_sensitivity_analysis</x:v>
+        <x:v>validate_constraints</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" hidden="0" customHeight="1">
-      <x:c r="A11" s="18" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B11" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="C11" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="D11" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E11" s="18" t="str">
-        <x:v>Monte Carlo不确定度分析</x:v>
-      </x:c>
-      <x:c r="F11" s="18" t="str">
-        <x:v>输入分布采样+模型批量执行</x:v>
-      </x:c>
-      <x:c r="G11" s="18" t="str">
-        <x:v>模型、输入分布、相关性、样本数</x:v>
-      </x:c>
-      <x:c r="H11" s="18" t="str">
-        <x:v>输出分布、区间、失效概率</x:v>
-      </x:c>
-      <x:c r="I11" s="18" t="str">
-        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
-      </x:c>
-      <x:c r="J11" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K11" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L11" s="18" t="str">
-        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
-      </x:c>
-      <x:c r="M11" s="18" t="str">
-        <x:v>A010,G006</x:v>
-      </x:c>
-      <x:c r="N11" s="18" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="O11" s="18" t="str">
-        <x:v>离线不确定度分析</x:v>
-      </x:c>
-      <x:c r="P11" s="18" t="str">
-        <x:v>run_monte_carlo_uncertainty</x:v>
-      </x:c>
+      <x:c r="A11" s="18"/>
+      <x:c r="B11" s="18"/>
+      <x:c r="C11" s="18"/>
+      <x:c r="D11" s="18"/>
+      <x:c r="E11" s="18"/>
+      <x:c r="F11" s="18"/>
+      <x:c r="G11" s="18"/>
+      <x:c r="H11" s="18"/>
+      <x:c r="I11" s="18"/>
+      <x:c r="J11" s="18"/>
+      <x:c r="K11" s="18"/>
+      <x:c r="L11" s="18"/>
+      <x:c r="M11" s="18"/>
+      <x:c r="N11" s="18"/>
+      <x:c r="O11" s="18"/>
+      <x:c r="P11" s="18"/>
     </x:row>
     <x:row r="12" ht="42" hidden="0" customHeight="1">
-      <x:c r="A12" s="18" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B12" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="C12" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="D12" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E12" s="18" t="str">
-        <x:v>贝叶斯优化</x:v>
-      </x:c>
-      <x:c r="F12" s="18" t="str">
-        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
-      </x:c>
-      <x:c r="G12" s="18" t="str">
-        <x:v>目标函数、约束、变量范围、预算</x:v>
-      </x:c>
-      <x:c r="H12" s="18" t="str">
-        <x:v>推荐下一组参数、最优历史、置信度</x:v>
-      </x:c>
-      <x:c r="I12" s="18" t="str">
-        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
-      </x:c>
-      <x:c r="J12" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K12" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L12" s="18" t="str">
-        <x:v>高斯过程/TPE采集函数</x:v>
-      </x:c>
-      <x:c r="M12" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N12" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O12" s="18" t="str">
-        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
-      </x:c>
-      <x:c r="P12" s="18" t="str">
-        <x:v>run_bayesian_optimization</x:v>
-      </x:c>
+      <x:c r="A12" s="18"/>
+      <x:c r="B12" s="18"/>
+      <x:c r="C12" s="18"/>
+      <x:c r="D12" s="18"/>
+      <x:c r="E12" s="18"/>
+      <x:c r="F12" s="18"/>
+      <x:c r="G12" s="18"/>
+      <x:c r="H12" s="18"/>
+      <x:c r="I12" s="18"/>
+      <x:c r="J12" s="18"/>
+      <x:c r="K12" s="18"/>
+      <x:c r="L12" s="18"/>
+      <x:c r="M12" s="18"/>
+      <x:c r="N12" s="18"/>
+      <x:c r="O12" s="18"/>
+      <x:c r="P12" s="18"/>
     </x:row>
     <x:row r="13" ht="42" hidden="0" customHeight="1">
-      <x:c r="A13" s="18" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B13" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="C13" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="D13" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E13" s="18" t="str">
-        <x:v>多目标优化</x:v>
-      </x:c>
-      <x:c r="F13" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="G13" s="18" t="str">
-        <x:v>目标、约束、变量、权重偏好</x:v>
-      </x:c>
-      <x:c r="H13" s="18" t="str">
-        <x:v>Pareto解集、折中解、约束状态</x:v>
-      </x:c>
-      <x:c r="I13" s="18" t="str">
-        <x:v>显式目标、约束、变量范围和偏好</x:v>
-      </x:c>
-      <x:c r="J13" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K13" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L13" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="M13" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N13" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O13" s="18" t="str">
-        <x:v>不读取企业历史数据</x:v>
-      </x:c>
-      <x:c r="P13" s="18" t="str">
-        <x:v>run_multiobjective_optimization</x:v>
-      </x:c>
+      <x:c r="A13" s="18"/>
+      <x:c r="B13" s="18"/>
+      <x:c r="C13" s="18"/>
+      <x:c r="D13" s="18"/>
+      <x:c r="E13" s="18"/>
+      <x:c r="F13" s="18"/>
+      <x:c r="G13" s="18"/>
+      <x:c r="H13" s="18"/>
+      <x:c r="I13" s="18"/>
+      <x:c r="J13" s="18"/>
+      <x:c r="K13" s="18"/>
+      <x:c r="L13" s="18"/>
+      <x:c r="M13" s="18"/>
+      <x:c r="N13" s="18"/>
+      <x:c r="O13" s="18"/>
+      <x:c r="P13" s="18"/>
     </x:row>
     <x:row r="14" ht="42" hidden="0" customHeight="1">
-      <x:c r="A14" s="18" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B14" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="C14" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="D14" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E14" s="18" t="str">
-        <x:v>约束规则校验器</x:v>
-      </x:c>
-      <x:c r="F14" s="18" t="str">
-        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="G14" s="18" t="str">
-        <x:v>模型输入输出、上下文、规则版本</x:v>
-      </x:c>
-      <x:c r="H14" s="18" t="str">
-        <x:v>通过/失败、违反规则、修复建议</x:v>
-      </x:c>
-      <x:c r="I14" s="18" t="str">
-        <x:v>显式模型输入输出与版本化JSON规则</x:v>
-      </x:c>
-      <x:c r="J14" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K14" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L14" s="18" t="str">
-        <x:v>表达式树、物料/能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="M14" s="18" t="str">
-        <x:v>A005</x:v>
-      </x:c>
-      <x:c r="N14" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O14" s="18" t="str">
-        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
-      </x:c>
-      <x:c r="P14" s="18" t="str">
-        <x:v>validate_constraints</x:v>
-      </x:c>
+      <x:c r="A14" s="18"/>
+      <x:c r="B14" s="18"/>
+      <x:c r="C14" s="18"/>
+      <x:c r="D14" s="18"/>
+      <x:c r="E14" s="18"/>
+      <x:c r="F14" s="18"/>
+      <x:c r="G14" s="18"/>
+      <x:c r="H14" s="18"/>
+      <x:c r="I14" s="18"/>
+      <x:c r="J14" s="18"/>
+      <x:c r="K14" s="18"/>
+      <x:c r="L14" s="18"/>
+      <x:c r="M14" s="18"/>
+      <x:c r="N14" s="18"/>
+      <x:c r="O14" s="18"/>
+      <x:c r="P14" s="18"/>
     </x:row>
     <x:row r="15" ht="42" hidden="0" customHeight="1">
       <x:c r="A15" s="18"/>
@@ -2488,7 +2360,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R074b8d7d6b834e89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R580b7e541aed43ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7208,10 +7080,10 @@
         <x:v>二冷分区水量分配</x:v>
       </x:c>
       <x:c r="D94" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E94" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W16</x:v>
       </x:c>
       <x:c r="F94" s="18" t="str">
         <x:v>F009</x:v>
@@ -7223,7 +7095,7 @@
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="I94" s="18" t="str">
-        <x:v>显式总水量、分区几何、喷嘴能力和温度约束</x:v>
+        <x:v>显式总水量、分区热需求、水量上下限和水侧热物性</x:v>
       </x:c>
       <x:c r="J94" s="18" t="str">
         <x:v>否</x:v>
@@ -7232,10 +7104,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L94" s="18" t="str">
-        <x:v>planned.f009.v1</x:v>
+        <x:v>metallurgy.catalog.f009.secondary_cooling_zone_allocation.v1</x:v>
       </x:c>
       <x:c r="M94" s="18" t="str">
-        <x:v>作为离线方案，不连接阀门或PLC</x:v>
+        <x:v>有界比例投影与显热校核；离线方案，不连接阀门或PLC</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="42" hidden="0" customHeight="1">
@@ -7249,10 +7121,10 @@
         <x:v>拉速优化</x:v>
       </x:c>
       <x:c r="D95" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E95" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W16</x:v>
       </x:c>
       <x:c r="F95" s="18" t="str">
         <x:v>F011</x:v>
@@ -7264,7 +7136,7 @@
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="I95" s="18" t="str">
-        <x:v>显式设备长度、温度/凝固约束与候选拉速区间</x:v>
+        <x:v>显式设备、停留时间、坯壳平方根律和冷却功率约束</x:v>
       </x:c>
       <x:c r="J95" s="18" t="str">
         <x:v>否</x:v>
@@ -7273,10 +7145,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L95" s="18" t="str">
-        <x:v>planned.f011.v1</x:v>
+        <x:v>metallurgy.catalog.f011.maximum_feasible_casting_speed.v1</x:v>
       </x:c>
       <x:c r="M95" s="18" t="str">
-        <x:v>不使用历史质量标签，不直接下发拉速</x:v>
+        <x:v>解析求最大可行拉速；不使用历史质量标签，不直接下发拉速</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="42" hidden="0" customHeight="1">
@@ -7290,10 +7162,10 @@
         <x:v>铸坯热应力/应变</x:v>
       </x:c>
       <x:c r="D96" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E96" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W16</x:v>
       </x:c>
       <x:c r="F96" s="18" t="str">
         <x:v>F014</x:v>
@@ -7305,7 +7177,7 @@
         <x:v>连铸质量与二冷</x:v>
       </x:c>
       <x:c r="I96" s="18" t="str">
-        <x:v>显式温度场、材料高温力学参数和边界条件</x:v>
+        <x:v>显式分层温度、模量、热膨胀系数、屈服和约束模式</x:v>
       </x:c>
       <x:c r="J96" s="18" t="str">
         <x:v>否</x:v>
@@ -7314,10 +7186,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L96" s="18" t="str">
-        <x:v>planned.f014.v1</x:v>
+        <x:v>metallurgy.catalog.f014.layered_thermal_stress.v1</x:v>
       </x:c>
       <x:c r="M96" s="18" t="str">
-        <x:v>不需要现场测温；仅分析显式温度场</x:v>
+        <x:v>一维平面应力弹性—理想塑性；不声称裂纹预测或有限元</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="42" hidden="0" customHeight="1">
@@ -7372,10 +7244,10 @@
         <x:v>一维传热PDE求解</x:v>
       </x:c>
       <x:c r="D98" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E98" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W16</x:v>
       </x:c>
       <x:c r="F98" s="18" t="str">
         <x:v>G003</x:v>
@@ -7387,7 +7259,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I98" s="18" t="str">
-        <x:v>显式几何、物性、热源和初边值</x:v>
+        <x:v>显式几何、常物性、热源、初温、边界和稳定时间步</x:v>
       </x:c>
       <x:c r="J98" s="18" t="str">
         <x:v>否</x:v>
@@ -7396,10 +7268,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L98" s="18" t="str">
-        <x:v>planned.g003.v1</x:v>
+        <x:v>metallurgy.catalog.g003.one_dimensional_heat_pde.v1</x:v>
       </x:c>
       <x:c r="M98" s="18" t="str">
-        <x:v>纯数值PDE，不使用现场数据</x:v>
+        <x:v>显式单元中心有限体积与能量闭合；不处理相变或温变物性</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="42" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
docs(tools): sync 120-tool catalog to 113 implemented
</commit_message>
<xml_diff>
--- a/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
+++ b/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rea36d924c4df4fb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R52046e73d1814c02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留9" sheetId="3" r:id="R40fc0ca356914585"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R0ee28584436743f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R51e60a944a214602"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rdcb93af001ab4bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R8a6ecf5095034e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留5" sheetId="3" r:id="Raa31c828f97b45a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R89944643a66f439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R0050bff17a5d4d5e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -533,7 +533,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>基线：main @ b861071；P1-W16新增F009、F011、F014、G003共4项后已实现109项，既有105项实现保持原样。</x:v>
+        <x:v>基线：main @ 93003d1；P1-W17新增G004、G008、G009、G010共4项后已实现113项，既有109项实现保持原样。</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -564,10 +564,10 @@
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:f>COUNTIF('最终120路线'!$D$2:$D$121,"已实现")</x:f>
-        <x:v>109</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>1. 已实现109项不改ID、不撤销资格；P1-W16新增F009、F011、F014、G003共4项。</x:v>
+        <x:v>1. 已实现113项不改ID、不撤销资格；P1-W17新增G004、G008、G009、G010共4项。</x:v>
       </x:c>
       <x:c r="E6" s="27"/>
       <x:c r="F6" s="27"/>
@@ -580,7 +580,7 @@
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:f>COUNTIFS('最终120路线'!$D$2:$D$121,"已实现",'最终120路线'!$G$2:$G$121,"是")</x:f>
-        <x:v>91</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
         <x:v>2. 延期项不注册、不生成空Schema、不计入count_eligible。</x:v>
@@ -596,7 +596,7 @@
       </x:c>
       <x:c r="B8" s="20" t="n">
         <x:f>120-B7</x:f>
-        <x:v>29</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>3. 后续工具不得以DS042、现场时序、企业标签或本地训练权重为准入前提。</x:v>
@@ -627,8 +627,8 @@
         <x:v>后续保留并去现场化</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:f>COUNTA('后续保留9'!$A$2:$A$10)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTA('后续保留5'!$A$2:$A$6)</x:f>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D10" s="27" t="str">
         <x:v>5. 允许使用公开算法、批准数据库和仓库内版本化常数。</x:v>
@@ -660,7 +660,7 @@
       </x:c>
       <x:c r="B12" s="20" t="n">
         <x:f>B10+B11</x:f>
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
         <x:v>7. 任何未来恢复的现场模型必须另行完成数据授权、脱敏和时序验证。</x:v>
@@ -681,7 +681,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>计数闭合：109 已实现 + 9 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
+        <x:v>计数闭合：113 已实现 + 5 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
       </x:c>
       <x:c r="B15" s="31"/>
       <x:c r="C15" s="31"/>
@@ -1495,28 +1495,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
-        <x:v>G004</x:v>
+        <x:v>G005</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
-        <x:v>反应ODE求解</x:v>
+        <x:v>CFD参数化案例生成</x:v>
       </x:c>
       <x:c r="F2" s="18" t="str">
-        <x:v>刚性/非刚性ODE自适应积分</x:v>
+        <x:v>模板渲染+参数/边界条件校验</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
-        <x:v>反应网络、速率、初值、时间区间</x:v>
+        <x:v>几何模板、物性、工况、求解器设置</x:v>
       </x:c>
       <x:c r="H2" s="18" t="str">
-        <x:v>状态轨迹、事件、收敛信息</x:v>
+        <x:v>可运行CFD案例目录、manifest</x:v>
       </x:c>
       <x:c r="I2" s="18" t="str">
-        <x:v>显式反应网络、速率表达式和初值</x:v>
+        <x:v>调用方显式提交几何模板、物性和工况</x:v>
       </x:c>
       <x:c r="J2" s="18" t="str">
         <x:v>否</x:v>
@@ -1525,19 +1525,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L2" s="18" t="str">
-        <x:v>自适应刚性/非刚性ODE积分</x:v>
+        <x:v>OpenFOAM案例模板与schema校验</x:v>
       </x:c>
       <x:c r="M2" s="18" t="str">
-        <x:v>C001,G002</x:v>
+        <x:v>G001,G002,G013</x:v>
       </x:c>
       <x:c r="N2" s="18" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O2" s="18" t="str">
-        <x:v>纯数值求解，不训练</x:v>
+        <x:v>DS042从必需来源中删除</x:v>
       </x:c>
       <x:c r="P2" s="18" t="str">
-        <x:v>solve_reaction_ode</x:v>
+        <x:v>generate_cfd_case</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
@@ -1545,28 +1545,28 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="C3" s="18" t="str">
-        <x:v>G005</x:v>
+        <x:v>G006</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
-        <x:v>CFD参数化案例生成</x:v>
+        <x:v>参数化仿真批处理</x:v>
       </x:c>
       <x:c r="F3" s="18" t="str">
-        <x:v>模板渲染+参数/边界条件校验</x:v>
+        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
-        <x:v>几何模板、物性、工况、求解器设置</x:v>
+        <x:v>案例模板、参数空间、资源配额</x:v>
       </x:c>
       <x:c r="H3" s="18" t="str">
-        <x:v>可运行CFD案例目录、manifest</x:v>
+        <x:v>运行状态、结果索引、失败原因</x:v>
       </x:c>
       <x:c r="I3" s="18" t="str">
-        <x:v>调用方显式提交几何模板、物性和工况</x:v>
+        <x:v>显式参数空间、案例模板和资源配额</x:v>
       </x:c>
       <x:c r="J3" s="18" t="str">
         <x:v>否</x:v>
@@ -1575,19 +1575,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L3" s="18" t="str">
-        <x:v>OpenFOAM案例模板与schema校验</x:v>
+        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
       </x:c>
       <x:c r="M3" s="18" t="str">
-        <x:v>G001,G002,G013</x:v>
+        <x:v>G005,G013</x:v>
       </x:c>
       <x:c r="N3" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O3" s="18" t="str">
-        <x:v>DS042从必需来源中删除</x:v>
+        <x:v>不读取现场数据；只编排批准案例</x:v>
       </x:c>
       <x:c r="P3" s="18" t="str">
-        <x:v>generate_cfd_case</x:v>
+        <x:v>run_parametric_simulation_batch</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" hidden="0" customHeight="1">
@@ -1595,28 +1595,28 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>G006</x:v>
+        <x:v>G011</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>参数化仿真批处理</x:v>
+        <x:v>贝叶斯优化</x:v>
       </x:c>
       <x:c r="F4" s="18" t="str">
-        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
+        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
       </x:c>
       <x:c r="G4" s="18" t="str">
-        <x:v>案例模板、参数空间、资源配额</x:v>
+        <x:v>目标函数、约束、变量范围、预算</x:v>
       </x:c>
       <x:c r="H4" s="18" t="str">
-        <x:v>运行状态、结果索引、失败原因</x:v>
+        <x:v>推荐下一组参数、最优历史、置信度</x:v>
       </x:c>
       <x:c r="I4" s="18" t="str">
-        <x:v>显式参数空间、案例模板和资源配额</x:v>
+        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
       </x:c>
       <x:c r="J4" s="18" t="str">
         <x:v>否</x:v>
@@ -1625,19 +1625,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L4" s="18" t="str">
-        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
+        <x:v>高斯过程/TPE采集函数</x:v>
       </x:c>
       <x:c r="M4" s="18" t="str">
-        <x:v>G005,G013</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N4" s="18" t="str">
         <x:v>高</x:v>
       </x:c>
       <x:c r="O4" s="18" t="str">
-        <x:v>不读取现场数据；只编排批准案例</x:v>
+        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
       </x:c>
       <x:c r="P4" s="18" t="str">
-        <x:v>run_parametric_simulation_batch</x:v>
+        <x:v>run_bayesian_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" hidden="0" customHeight="1">
@@ -1645,28 +1645,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>G008</x:v>
+        <x:v>G012</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>插值与查表服务</x:v>
+        <x:v>多目标优化</x:v>
       </x:c>
       <x:c r="F5" s="18" t="str">
-        <x:v>多维规则网格/散点插值+缓存</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="G5" s="18" t="str">
-        <x:v>查询点、表格版本、外推策略</x:v>
+        <x:v>目标、约束、变量、权重偏好</x:v>
       </x:c>
       <x:c r="H5" s="18" t="str">
-        <x:v>插值值、距离、是否外推</x:v>
+        <x:v>Pareto解集、折中解、约束状态</x:v>
       </x:c>
       <x:c r="I5" s="18" t="str">
-        <x:v>调用方上传或选择版本化查找表</x:v>
+        <x:v>显式目标、约束、变量范围和偏好</x:v>
       </x:c>
       <x:c r="J5" s="18" t="str">
         <x:v>否</x:v>
@@ -1675,19 +1675,19 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L5" s="18" t="str">
-        <x:v>规则网格/散点插值和外推距离</x:v>
+        <x:v>NSGA-II/ε约束/Pyomo</x:v>
       </x:c>
       <x:c r="M5" s="18" t="str">
-        <x:v>A004</x:v>
+        <x:v>G009,G013</x:v>
       </x:c>
       <x:c r="N5" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O5" s="18" t="str">
-        <x:v>不连接企业实时表</x:v>
+        <x:v>不读取企业历史数据</x:v>
       </x:c>
       <x:c r="P5" s="18" t="str">
-        <x:v>interpolate_lookup_table</x:v>
+        <x:v>run_multiobjective_optimization</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" hidden="0" customHeight="1">
@@ -1695,28 +1695,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>G009</x:v>
+        <x:v>G013</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>敏感性分析</x:v>
+        <x:v>约束规则校验器</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol可选</x:v>
+        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
-        <x:v>模型、参数范围、采样预算</x:v>
+        <x:v>模型输入输出、上下文、规则版本</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
-        <x:v>敏感度排序、交互效应</x:v>
+        <x:v>通过/失败、违反规则、修复建议</x:v>
       </x:c>
       <x:c r="I6" s="18" t="str">
-        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
+        <x:v>显式模型输入输出与版本化JSON规则</x:v>
       </x:c>
       <x:c r="J6" s="18" t="str">
         <x:v>否</x:v>
@@ -1725,220 +1725,92 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L6" s="18" t="str">
-        <x:v>局部导数、Morris/Sobol</x:v>
+        <x:v>表达式树、物料/能量与工艺边界</x:v>
       </x:c>
       <x:c r="M6" s="18" t="str">
-        <x:v>A010,G008</x:v>
+        <x:v>A005</x:v>
       </x:c>
       <x:c r="N6" s="18" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="O6" s="18" t="str">
-        <x:v>离线分析，不使用历史成功率</x:v>
+        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
       </x:c>
       <x:c r="P6" s="18" t="str">
-        <x:v>run_sensitivity_analysis</x:v>
+        <x:v>validate_constraints</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" hidden="0" customHeight="1">
-      <x:c r="A7" s="18" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B7" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="C7" s="18" t="str">
-        <x:v>G010</x:v>
-      </x:c>
-      <x:c r="D7" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E7" s="18" t="str">
-        <x:v>Monte Carlo不确定度分析</x:v>
-      </x:c>
-      <x:c r="F7" s="18" t="str">
-        <x:v>输入分布采样+模型批量执行</x:v>
-      </x:c>
-      <x:c r="G7" s="18" t="str">
-        <x:v>模型、输入分布、相关性、样本数</x:v>
-      </x:c>
-      <x:c r="H7" s="18" t="str">
-        <x:v>输出分布、区间、失效概率</x:v>
-      </x:c>
-      <x:c r="I7" s="18" t="str">
-        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
-      </x:c>
-      <x:c r="J7" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K7" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L7" s="18" t="str">
-        <x:v>固定种子Monte Carlo与收敛诊断</x:v>
-      </x:c>
-      <x:c r="M7" s="18" t="str">
-        <x:v>A010,G006</x:v>
-      </x:c>
-      <x:c r="N7" s="18" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="O7" s="18" t="str">
-        <x:v>离线不确定度分析</x:v>
-      </x:c>
-      <x:c r="P7" s="18" t="str">
-        <x:v>run_monte_carlo_uncertainty</x:v>
-      </x:c>
+      <x:c r="A7" s="18"/>
+      <x:c r="B7" s="18"/>
+      <x:c r="C7" s="18"/>
+      <x:c r="D7" s="18"/>
+      <x:c r="E7" s="18"/>
+      <x:c r="F7" s="18"/>
+      <x:c r="G7" s="18"/>
+      <x:c r="H7" s="18"/>
+      <x:c r="I7" s="18"/>
+      <x:c r="J7" s="18"/>
+      <x:c r="K7" s="18"/>
+      <x:c r="L7" s="18"/>
+      <x:c r="M7" s="18"/>
+      <x:c r="N7" s="18"/>
+      <x:c r="O7" s="18"/>
+      <x:c r="P7" s="18"/>
     </x:row>
     <x:row r="8" ht="42" hidden="0" customHeight="1">
-      <x:c r="A8" s="18" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B8" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="C8" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="D8" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E8" s="18" t="str">
-        <x:v>贝叶斯优化</x:v>
-      </x:c>
-      <x:c r="F8" s="18" t="str">
-        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
-      </x:c>
-      <x:c r="G8" s="18" t="str">
-        <x:v>目标函数、约束、变量范围、预算</x:v>
-      </x:c>
-      <x:c r="H8" s="18" t="str">
-        <x:v>推荐下一组参数、最优历史、置信度</x:v>
-      </x:c>
-      <x:c r="I8" s="18" t="str">
-        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
-      </x:c>
-      <x:c r="J8" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K8" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L8" s="18" t="str">
-        <x:v>高斯过程/TPE采集函数</x:v>
-      </x:c>
-      <x:c r="M8" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N8" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O8" s="18" t="str">
-        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
-      </x:c>
-      <x:c r="P8" s="18" t="str">
-        <x:v>run_bayesian_optimization</x:v>
-      </x:c>
+      <x:c r="A8" s="18"/>
+      <x:c r="B8" s="18"/>
+      <x:c r="C8" s="18"/>
+      <x:c r="D8" s="18"/>
+      <x:c r="E8" s="18"/>
+      <x:c r="F8" s="18"/>
+      <x:c r="G8" s="18"/>
+      <x:c r="H8" s="18"/>
+      <x:c r="I8" s="18"/>
+      <x:c r="J8" s="18"/>
+      <x:c r="K8" s="18"/>
+      <x:c r="L8" s="18"/>
+      <x:c r="M8" s="18"/>
+      <x:c r="N8" s="18"/>
+      <x:c r="O8" s="18"/>
+      <x:c r="P8" s="18"/>
     </x:row>
     <x:row r="9" ht="42" hidden="0" customHeight="1">
-      <x:c r="A9" s="18" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B9" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="C9" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="D9" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E9" s="18" t="str">
-        <x:v>多目标优化</x:v>
-      </x:c>
-      <x:c r="F9" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="G9" s="18" t="str">
-        <x:v>目标、约束、变量、权重偏好</x:v>
-      </x:c>
-      <x:c r="H9" s="18" t="str">
-        <x:v>Pareto解集、折中解、约束状态</x:v>
-      </x:c>
-      <x:c r="I9" s="18" t="str">
-        <x:v>显式目标、约束、变量范围和偏好</x:v>
-      </x:c>
-      <x:c r="J9" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K9" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L9" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="M9" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N9" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O9" s="18" t="str">
-        <x:v>不读取企业历史数据</x:v>
-      </x:c>
-      <x:c r="P9" s="18" t="str">
-        <x:v>run_multiobjective_optimization</x:v>
-      </x:c>
+      <x:c r="A9" s="18"/>
+      <x:c r="B9" s="18"/>
+      <x:c r="C9" s="18"/>
+      <x:c r="D9" s="18"/>
+      <x:c r="E9" s="18"/>
+      <x:c r="F9" s="18"/>
+      <x:c r="G9" s="18"/>
+      <x:c r="H9" s="18"/>
+      <x:c r="I9" s="18"/>
+      <x:c r="J9" s="18"/>
+      <x:c r="K9" s="18"/>
+      <x:c r="L9" s="18"/>
+      <x:c r="M9" s="18"/>
+      <x:c r="N9" s="18"/>
+      <x:c r="O9" s="18"/>
+      <x:c r="P9" s="18"/>
     </x:row>
     <x:row r="10" ht="42" hidden="0" customHeight="1">
-      <x:c r="A10" s="18" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B10" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="C10" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="D10" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E10" s="18" t="str">
-        <x:v>约束规则校验器</x:v>
-      </x:c>
-      <x:c r="F10" s="18" t="str">
-        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="G10" s="18" t="str">
-        <x:v>模型输入输出、上下文、规则版本</x:v>
-      </x:c>
-      <x:c r="H10" s="18" t="str">
-        <x:v>通过/失败、违反规则、修复建议</x:v>
-      </x:c>
-      <x:c r="I10" s="18" t="str">
-        <x:v>显式模型输入输出与版本化JSON规则</x:v>
-      </x:c>
-      <x:c r="J10" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K10" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L10" s="18" t="str">
-        <x:v>表达式树、物料/能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="M10" s="18" t="str">
-        <x:v>A005</x:v>
-      </x:c>
-      <x:c r="N10" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O10" s="18" t="str">
-        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
-      </x:c>
-      <x:c r="P10" s="18" t="str">
-        <x:v>validate_constraints</x:v>
-      </x:c>
+      <x:c r="A10" s="18"/>
+      <x:c r="B10" s="18"/>
+      <x:c r="C10" s="18"/>
+      <x:c r="D10" s="18"/>
+      <x:c r="E10" s="18"/>
+      <x:c r="F10" s="18"/>
+      <x:c r="G10" s="18"/>
+      <x:c r="H10" s="18"/>
+      <x:c r="I10" s="18"/>
+      <x:c r="J10" s="18"/>
+      <x:c r="K10" s="18"/>
+      <x:c r="L10" s="18"/>
+      <x:c r="M10" s="18"/>
+      <x:c r="N10" s="18"/>
+      <x:c r="O10" s="18"/>
+      <x:c r="P10" s="18"/>
     </x:row>
     <x:row r="11" ht="42" hidden="0" customHeight="1">
       <x:c r="A11" s="18"/>
@@ -2360,7 +2232,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R580b7e541aed43ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89c7234448574e91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7285,10 +7157,10 @@
         <x:v>反应ODE求解</x:v>
       </x:c>
       <x:c r="D99" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E99" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W17</x:v>
       </x:c>
       <x:c r="F99" s="18" t="str">
         <x:v>G004</x:v>
@@ -7300,7 +7172,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I99" s="18" t="str">
-        <x:v>显式反应网络、速率表达式和初值</x:v>
+        <x:v>显式反应网络、化学计量、初始浓度、时间和求解设置</x:v>
       </x:c>
       <x:c r="J99" s="18" t="str">
         <x:v>否</x:v>
@@ -7309,10 +7181,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L99" s="18" t="str">
-        <x:v>planned.g004.v1</x:v>
+        <x:v>metallurgy.catalog.g004.structured_mass_action_ode.v1</x:v>
       </x:c>
       <x:c r="M99" s="18" t="str">
-        <x:v>纯数值求解，不训练</x:v>
+        <x:v>结构化质量作用+solve_ivp；不接受任意表达式，不含传热传质</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="42" hidden="0" customHeight="1">
@@ -7408,10 +7280,10 @@
         <x:v>插值与查表服务</x:v>
       </x:c>
       <x:c r="D102" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E102" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W17</x:v>
       </x:c>
       <x:c r="F102" s="18" t="str">
         <x:v>G008</x:v>
@@ -7423,7 +7295,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I102" s="18" t="str">
-        <x:v>调用方上传或选择版本化查找表</x:v>
+        <x:v>显式一/二维规则表、表ID/版本/单位、查询点与边界策略</x:v>
       </x:c>
       <x:c r="J102" s="18" t="str">
         <x:v>否</x:v>
@@ -7432,10 +7304,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L102" s="18" t="str">
-        <x:v>planned.g008.v1</x:v>
+        <x:v>metallurgy.catalog.g008.regular_grid_lookup.v1</x:v>
       </x:c>
       <x:c r="M102" s="18" t="str">
-        <x:v>不连接企业实时表</x:v>
+        <x:v>线性/双线性/确定性最近邻；不连接企业实时表，不隐式外推</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="42" hidden="0" customHeight="1">
@@ -7449,10 +7321,10 @@
         <x:v>敏感性分析</x:v>
       </x:c>
       <x:c r="D103" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E103" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W17</x:v>
       </x:c>
       <x:c r="F103" s="18" t="str">
         <x:v>G009</x:v>
@@ -7464,7 +7336,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I103" s="18" t="str">
-        <x:v>显式模型函数、参数范围和固定采样方案</x:v>
+        <x:v>已认证目标工具、基准参数、标量输出路径和数值扰动步长</x:v>
       </x:c>
       <x:c r="J103" s="18" t="str">
         <x:v>否</x:v>
@@ -7473,10 +7345,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L103" s="18" t="str">
-        <x:v>planned.g009.v1</x:v>
+        <x:v>metallurgy.catalog.g009.registered_tool_local_sensitivity.v1</x:v>
       </x:c>
       <x:c r="M103" s="18" t="str">
-        <x:v>离线分析，不使用历史成功率</x:v>
+        <x:v>安全注册工具中心差分；局部结果不等同全局敏感性，不执行任意代码</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="42" hidden="0" customHeight="1">
@@ -7490,10 +7362,10 @@
         <x:v>Monte Carlo不确定度分析</x:v>
       </x:c>
       <x:c r="D104" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E104" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W17</x:v>
       </x:c>
       <x:c r="F104" s="18" t="str">
         <x:v>G010</x:v>
@@ -7505,7 +7377,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I104" s="18" t="str">
-        <x:v>显式概率分布、相关性、样本数和可调用模型</x:v>
+        <x:v>已认证目标工具、参数分布、相关矩阵、固定种子和样本数</x:v>
       </x:c>
       <x:c r="J104" s="18" t="str">
         <x:v>否</x:v>
@@ -7514,10 +7386,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L104" s="18" t="str">
-        <x:v>planned.g010.v1</x:v>
+        <x:v>metallurgy.catalog.g010.registered_tool_monte_carlo.v1</x:v>
       </x:c>
       <x:c r="M104" s="18" t="str">
-        <x:v>离线不确定度分析</x:v>
+        <x:v>固定种子Gaussian copula+注册工具传播；不连接现场数据，不用于稀有事件认证</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="42" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
feat(tools): complete qualified 120-tool registry
</commit_message>
<xml_diff>
--- a/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
+++ b/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rdcb93af001ab4bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="R8a6ecf5095034e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留5" sheetId="3" r:id="Raa31c828f97b45a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R89944643a66f439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R0050bff17a5d4d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R31f7ef06e1544f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="Raf39284d2c784b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留5" sheetId="3" r:id="R2846b9a4e8b94a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R202a3b95e8db4d14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="Rcd638e61da50497f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -533,7 +533,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>基线：main @ 93003d1；P1-W17新增G004、G008、G009、G010共4项后已实现113项，既有109项实现保持原样。</x:v>
+        <x:v>基线：main @ 60c2232；P1-W18新增并认证G005、G006、G011、G012、G013、E022、H001共7项后，120项均已实现并通过统一资格闸门。</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -564,10 +564,10 @@
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:f>COUNTIF('最终120路线'!$D$2:$D$121,"已实现")</x:f>
-        <x:v>113</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>1. 已实现113项不改ID、不撤销资格；P1-W17新增G004、G008、G009、G010共4项。</x:v>
+        <x:v>1. 120项真实工具均已实现、保留稳定ID并通过实现、数据、接口与科学验证四维资格闸门；P1-W18闭合最后7项。</x:v>
       </x:c>
       <x:c r="E6" s="27"/>
       <x:c r="F6" s="27"/>
@@ -580,7 +580,7 @@
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:f>COUNTIFS('最终120路线'!$D$2:$D$121,"已实现",'最终120路线'!$G$2:$G$121,"是")</x:f>
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
         <x:v>2. 延期项不注册、不生成空Schema、不计入count_eligible。</x:v>
@@ -596,7 +596,7 @@
       </x:c>
       <x:c r="B8" s="20" t="n">
         <x:f>120-B7</x:f>
-        <x:v>25</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
         <x:v>3. 后续工具不得以DS042、现场时序、企业标签或本地训练权重为准入前提。</x:v>
@@ -628,7 +628,7 @@
       </x:c>
       <x:c r="B10" s="20" t="n">
         <x:f>COUNTA('后续保留5'!$A$2:$A$6)</x:f>
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="27" t="str">
         <x:v>5. 允许使用公开算法、批准数据库和仓库内版本化常数。</x:v>
@@ -644,7 +644,7 @@
       </x:c>
       <x:c r="B11" s="20" t="n">
         <x:f>COUNTIF('最终120路线'!$D$2:$D$121,"新增替换")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D11" s="27" t="str">
         <x:v>6. 优化工具只输出离线方案，不直接下发PLC、设备或联锁。</x:v>
@@ -660,7 +660,7 @@
       </x:c>
       <x:c r="B12" s="20" t="n">
         <x:f>B10+B11</x:f>
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
         <x:v>7. 任何未来恢复的现场模型必须另行完成数据授权、脱敏和时序验证。</x:v>
@@ -681,7 +681,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>计数闭合：113 已实现 + 5 后续保留 + 2 剩余新增替换 = 120；20 项现场数据依赖能力进入延期池。</x:v>
+        <x:v>计数闭合：120 已实现 + 0 后续保留 + 0 剩余新增替换 = 120；20 项现场/训练数据依赖能力继续留在延期池，不注册、不计数。</x:v>
       </x:c>
       <x:c r="B15" s="31"/>
       <x:c r="C15" s="31"/>
@@ -1491,254 +1491,94 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="42" hidden="0" customHeight="1">
-      <x:c r="A2" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="18" t="str">
-        <x:v>G005</x:v>
-      </x:c>
-      <x:c r="C2" s="18" t="str">
-        <x:v>G005</x:v>
-      </x:c>
-      <x:c r="D2" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E2" s="18" t="str">
-        <x:v>CFD参数化案例生成</x:v>
-      </x:c>
-      <x:c r="F2" s="18" t="str">
-        <x:v>模板渲染+参数/边界条件校验</x:v>
-      </x:c>
-      <x:c r="G2" s="18" t="str">
-        <x:v>几何模板、物性、工况、求解器设置</x:v>
-      </x:c>
-      <x:c r="H2" s="18" t="str">
-        <x:v>可运行CFD案例目录、manifest</x:v>
-      </x:c>
-      <x:c r="I2" s="18" t="str">
-        <x:v>调用方显式提交几何模板、物性和工况</x:v>
-      </x:c>
-      <x:c r="J2" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K2" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L2" s="18" t="str">
-        <x:v>OpenFOAM案例模板与schema校验</x:v>
-      </x:c>
-      <x:c r="M2" s="18" t="str">
-        <x:v>G001,G002,G013</x:v>
-      </x:c>
-      <x:c r="N2" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O2" s="18" t="str">
-        <x:v>DS042从必需来源中删除</x:v>
-      </x:c>
-      <x:c r="P2" s="18" t="str">
-        <x:v>generate_cfd_case</x:v>
-      </x:c>
+      <x:c r="A2" s="18"/>
+      <x:c r="B2" s="18"/>
+      <x:c r="C2" s="18"/>
+      <x:c r="D2" s="18"/>
+      <x:c r="E2" s="18"/>
+      <x:c r="F2" s="18"/>
+      <x:c r="G2" s="18"/>
+      <x:c r="H2" s="18"/>
+      <x:c r="I2" s="18"/>
+      <x:c r="J2" s="18"/>
+      <x:c r="K2" s="18"/>
+      <x:c r="L2" s="18"/>
+      <x:c r="M2" s="18"/>
+      <x:c r="N2" s="18"/>
+      <x:c r="O2" s="18"/>
+      <x:c r="P2" s="18"/>
     </x:row>
     <x:row r="3" ht="42" hidden="0" customHeight="1">
-      <x:c r="A3" s="18" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="18" t="str">
-        <x:v>G006</x:v>
-      </x:c>
-      <x:c r="C3" s="18" t="str">
-        <x:v>G006</x:v>
-      </x:c>
-      <x:c r="D3" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E3" s="18" t="str">
-        <x:v>参数化仿真批处理</x:v>
-      </x:c>
-      <x:c r="F3" s="18" t="str">
-        <x:v>参数网格/试验设计+容器队列+失败重试</x:v>
-      </x:c>
-      <x:c r="G3" s="18" t="str">
-        <x:v>案例模板、参数空间、资源配额</x:v>
-      </x:c>
-      <x:c r="H3" s="18" t="str">
-        <x:v>运行状态、结果索引、失败原因</x:v>
-      </x:c>
-      <x:c r="I3" s="18" t="str">
-        <x:v>显式参数空间、案例模板和资源配额</x:v>
-      </x:c>
-      <x:c r="J3" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K3" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L3" s="18" t="str">
-        <x:v>可复现参数网格、运行manifest和失败重试</x:v>
-      </x:c>
-      <x:c r="M3" s="18" t="str">
-        <x:v>G005,G013</x:v>
-      </x:c>
-      <x:c r="N3" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O3" s="18" t="str">
-        <x:v>不读取现场数据；只编排批准案例</x:v>
-      </x:c>
-      <x:c r="P3" s="18" t="str">
-        <x:v>run_parametric_simulation_batch</x:v>
-      </x:c>
+      <x:c r="A3" s="18"/>
+      <x:c r="B3" s="18"/>
+      <x:c r="C3" s="18"/>
+      <x:c r="D3" s="18"/>
+      <x:c r="E3" s="18"/>
+      <x:c r="F3" s="18"/>
+      <x:c r="G3" s="18"/>
+      <x:c r="H3" s="18"/>
+      <x:c r="I3" s="18"/>
+      <x:c r="J3" s="18"/>
+      <x:c r="K3" s="18"/>
+      <x:c r="L3" s="18"/>
+      <x:c r="M3" s="18"/>
+      <x:c r="N3" s="18"/>
+      <x:c r="O3" s="18"/>
+      <x:c r="P3" s="18"/>
     </x:row>
     <x:row r="4" ht="42" hidden="0" customHeight="1">
-      <x:c r="A4" s="18" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B4" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="C4" s="18" t="str">
-        <x:v>G011</x:v>
-      </x:c>
-      <x:c r="D4" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E4" s="18" t="str">
-        <x:v>贝叶斯优化</x:v>
-      </x:c>
-      <x:c r="F4" s="18" t="str">
-        <x:v>离线贝叶斯优化；目标仅来自显式函数或已注册工具</x:v>
-      </x:c>
-      <x:c r="G4" s="18" t="str">
-        <x:v>目标函数、约束、变量范围、预算</x:v>
-      </x:c>
-      <x:c r="H4" s="18" t="str">
-        <x:v>推荐下一组参数、最优历史、置信度</x:v>
-      </x:c>
-      <x:c r="I4" s="18" t="str">
-        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
-      </x:c>
-      <x:c r="J4" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K4" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L4" s="18" t="str">
-        <x:v>高斯过程/TPE采集函数</x:v>
-      </x:c>
-      <x:c r="M4" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N4" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O4" s="18" t="str">
-        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
-      </x:c>
-      <x:c r="P4" s="18" t="str">
-        <x:v>run_bayesian_optimization</x:v>
-      </x:c>
+      <x:c r="A4" s="18"/>
+      <x:c r="B4" s="18"/>
+      <x:c r="C4" s="18"/>
+      <x:c r="D4" s="18"/>
+      <x:c r="E4" s="18"/>
+      <x:c r="F4" s="18"/>
+      <x:c r="G4" s="18"/>
+      <x:c r="H4" s="18"/>
+      <x:c r="I4" s="18"/>
+      <x:c r="J4" s="18"/>
+      <x:c r="K4" s="18"/>
+      <x:c r="L4" s="18"/>
+      <x:c r="M4" s="18"/>
+      <x:c r="N4" s="18"/>
+      <x:c r="O4" s="18"/>
+      <x:c r="P4" s="18"/>
     </x:row>
     <x:row r="5" ht="42" hidden="0" customHeight="1">
-      <x:c r="A5" s="18" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B5" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="C5" s="18" t="str">
-        <x:v>G012</x:v>
-      </x:c>
-      <x:c r="D5" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E5" s="18" t="str">
-        <x:v>多目标优化</x:v>
-      </x:c>
-      <x:c r="F5" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="G5" s="18" t="str">
-        <x:v>目标、约束、变量、权重偏好</x:v>
-      </x:c>
-      <x:c r="H5" s="18" t="str">
-        <x:v>Pareto解集、折中解、约束状态</x:v>
-      </x:c>
-      <x:c r="I5" s="18" t="str">
-        <x:v>显式目标、约束、变量范围和偏好</x:v>
-      </x:c>
-      <x:c r="J5" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K5" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L5" s="18" t="str">
-        <x:v>NSGA-II/ε约束/Pyomo</x:v>
-      </x:c>
-      <x:c r="M5" s="18" t="str">
-        <x:v>G009,G013</x:v>
-      </x:c>
-      <x:c r="N5" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O5" s="18" t="str">
-        <x:v>不读取企业历史数据</x:v>
-      </x:c>
-      <x:c r="P5" s="18" t="str">
-        <x:v>run_multiobjective_optimization</x:v>
-      </x:c>
+      <x:c r="A5" s="18"/>
+      <x:c r="B5" s="18"/>
+      <x:c r="C5" s="18"/>
+      <x:c r="D5" s="18"/>
+      <x:c r="E5" s="18"/>
+      <x:c r="F5" s="18"/>
+      <x:c r="G5" s="18"/>
+      <x:c r="H5" s="18"/>
+      <x:c r="I5" s="18"/>
+      <x:c r="J5" s="18"/>
+      <x:c r="K5" s="18"/>
+      <x:c r="L5" s="18"/>
+      <x:c r="M5" s="18"/>
+      <x:c r="N5" s="18"/>
+      <x:c r="O5" s="18"/>
+      <x:c r="P5" s="18"/>
     </x:row>
     <x:row r="6" ht="42" hidden="0" customHeight="1">
-      <x:c r="A6" s="18" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="C6" s="18" t="str">
-        <x:v>G013</x:v>
-      </x:c>
-      <x:c r="D6" s="18" t="str">
-        <x:v>仿真/优化/智能体支撑</x:v>
-      </x:c>
-      <x:c r="E6" s="18" t="str">
-        <x:v>约束规则校验器</x:v>
-      </x:c>
-      <x:c r="F6" s="18" t="str">
-        <x:v>JSON规则/表达式树/物料能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="G6" s="18" t="str">
-        <x:v>模型输入输出、上下文、规则版本</x:v>
-      </x:c>
-      <x:c r="H6" s="18" t="str">
-        <x:v>通过/失败、违反规则、修复建议</x:v>
-      </x:c>
-      <x:c r="I6" s="18" t="str">
-        <x:v>显式模型输入输出与版本化JSON规则</x:v>
-      </x:c>
-      <x:c r="J6" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K6" s="18" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L6" s="18" t="str">
-        <x:v>表达式树、物料/能量与工艺边界</x:v>
-      </x:c>
-      <x:c r="M6" s="18" t="str">
-        <x:v>A005</x:v>
-      </x:c>
-      <x:c r="N6" s="18" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="O6" s="18" t="str">
-        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
-      </x:c>
-      <x:c r="P6" s="18" t="str">
-        <x:v>validate_constraints</x:v>
-      </x:c>
+      <x:c r="A6" s="18"/>
+      <x:c r="B6" s="18"/>
+      <x:c r="C6" s="18"/>
+      <x:c r="D6" s="18"/>
+      <x:c r="E6" s="18"/>
+      <x:c r="F6" s="18"/>
+      <x:c r="G6" s="18"/>
+      <x:c r="H6" s="18"/>
+      <x:c r="I6" s="18"/>
+      <x:c r="J6" s="18"/>
+      <x:c r="K6" s="18"/>
+      <x:c r="L6" s="18"/>
+      <x:c r="M6" s="18"/>
+      <x:c r="N6" s="18"/>
+      <x:c r="O6" s="18"/>
+      <x:c r="P6" s="18"/>
     </x:row>
     <x:row r="7" ht="42" hidden="0" customHeight="1">
       <x:c r="A7" s="18"/>
@@ -2232,7 +2072,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89c7234448574e91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0b21bb605dc4b34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7195,13 +7035,13 @@
         <x:v>G005</x:v>
       </x:c>
       <x:c r="C100" s="18" t="str">
-        <x:v>CFD参数化案例生成</x:v>
+        <x:v>OpenFOAM参数化导热案例生成</x:v>
       </x:c>
       <x:c r="D100" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E100" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W18</x:v>
       </x:c>
       <x:c r="F100" s="18" t="str">
         <x:v>G005</x:v>
@@ -7213,7 +7053,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I100" s="18" t="str">
-        <x:v>调用方显式提交几何模板、物性和工况</x:v>
+        <x:v>显式长方体几何、网格、扩散率、边界与时间设置；仅生成OpenFOAM v13清单</x:v>
       </x:c>
       <x:c r="J100" s="18" t="str">
         <x:v>否</x:v>
@@ -7222,10 +7062,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L100" s="18" t="str">
-        <x:v>planned.g005.v1</x:v>
+        <x:v>metallurgy.catalog.g005.openfoam_laplacian_case.v1</x:v>
       </x:c>
       <x:c r="M100" s="18" t="str">
-        <x:v>DS042从必需来源中删除</x:v>
+        <x:v>受限laplacianFoam案例清单；不写任意路径、不执行求解器</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="42" hidden="0" customHeight="1">
@@ -7236,13 +7076,13 @@
         <x:v>G006</x:v>
       </x:c>
       <x:c r="C101" s="18" t="str">
-        <x:v>参数化仿真批处理</x:v>
+        <x:v>注册工具参数化仿真批处理</x:v>
       </x:c>
       <x:c r="D101" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E101" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W18</x:v>
       </x:c>
       <x:c r="F101" s="18" t="str">
         <x:v>G006</x:v>
@@ -7254,7 +7094,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I101" s="18" t="str">
-        <x:v>显式参数空间、案例模板和资源配额</x:v>
+        <x:v>完全准入目标工具、显式基础参数、数值参数网格、配额与重试策略</x:v>
       </x:c>
       <x:c r="J101" s="18" t="str">
         <x:v>否</x:v>
@@ -7263,10 +7103,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L101" s="18" t="str">
-        <x:v>planned.g006.v1</x:v>
+        <x:v>metallurgy.catalog.g006.registered_parametric_batch.v1</x:v>
       </x:c>
       <x:c r="M101" s="18" t="str">
-        <x:v>不读取现场数据；只编排批准案例</x:v>
+        <x:v>确定性笛卡尔参数批处理；只调用统一注册中心，不执行shell</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="42" hidden="0" customHeight="1">
@@ -7400,13 +7240,13 @@
         <x:v>G011</x:v>
       </x:c>
       <x:c r="C105" s="18" t="str">
-        <x:v>贝叶斯优化</x:v>
+        <x:v>离线高斯过程贝叶斯优化</x:v>
       </x:c>
       <x:c r="D105" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E105" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W18</x:v>
       </x:c>
       <x:c r="F105" s="18" t="str">
         <x:v>G011</x:v>
@@ -7418,7 +7258,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I105" s="18" t="str">
-        <x:v>显式变量域、目标函数、约束和评估预算</x:v>
+        <x:v>完全准入目标工具、连续变量域、标量目标、显式约束、预算与固定种子</x:v>
       </x:c>
       <x:c r="J105" s="18" t="str">
         <x:v>否</x:v>
@@ -7427,10 +7267,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L105" s="18" t="str">
-        <x:v>planned.g011.v1</x:v>
+        <x:v>metallurgy.catalog.g011.offline_gp_expected_improvement.v1</x:v>
       </x:c>
       <x:c r="M105" s="18" t="str">
-        <x:v>‘在线’改为离线序贯评估，不连接生产过程</x:v>
+        <x:v>固定RBF高斯过程与Expected Improvement；离线序贯评估，不连接生产过程</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="42" hidden="0" customHeight="1">
@@ -7441,13 +7281,13 @@
         <x:v>G012</x:v>
       </x:c>
       <x:c r="C106" s="18" t="str">
-        <x:v>多目标优化</x:v>
+        <x:v>注册工具NSGA-II多目标优化</x:v>
       </x:c>
       <x:c r="D106" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E106" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W18</x:v>
       </x:c>
       <x:c r="F106" s="18" t="str">
         <x:v>G012</x:v>
@@ -7459,7 +7299,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I106" s="18" t="str">
-        <x:v>显式目标、约束、变量范围和偏好</x:v>
+        <x:v>完全准入目标工具、连续变量、2至4个目标、显式约束、种群/代数与固定种子</x:v>
       </x:c>
       <x:c r="J106" s="18" t="str">
         <x:v>否</x:v>
@@ -7468,10 +7308,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L106" s="18" t="str">
-        <x:v>planned.g012.v1</x:v>
+        <x:v>metallurgy.catalog.g012.constrained_nsga2.v1</x:v>
       </x:c>
       <x:c r="M106" s="18" t="str">
-        <x:v>不读取企业历史数据</x:v>
+        <x:v>约束NSGA-II、非支配集与透明折中解；不读取企业历史数据</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="42" hidden="0" customHeight="1">
@@ -7482,13 +7322,13 @@
         <x:v>G013</x:v>
       </x:c>
       <x:c r="C107" s="18" t="str">
-        <x:v>约束规则校验器</x:v>
+        <x:v>安全约束规则校验器</x:v>
       </x:c>
       <x:c r="D107" s="18" t="str">
-        <x:v>后续保留</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E107" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W18</x:v>
       </x:c>
       <x:c r="F107" s="18" t="str">
         <x:v>G013</x:v>
@@ -7500,7 +7340,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I107" s="18" t="str">
-        <x:v>显式模型输入输出与版本化JSON规则</x:v>
+        <x:v>显式JSON上下文、规则集ID/版本和受限表达式树</x:v>
       </x:c>
       <x:c r="J107" s="18" t="str">
         <x:v>否</x:v>
@@ -7509,10 +7349,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L107" s="18" t="str">
-        <x:v>planned.g013.v1</x:v>
+        <x:v>metallurgy.catalog.g013.safe_versioned_constraints.v1</x:v>
       </x:c>
       <x:c r="M107" s="18" t="str">
-        <x:v>规则由仓库版本化，不从专家历史自动学习</x:v>
+        <x:v>仅允许白名单表达式节点；不eval、不导入模块、不访问文件/网络/数据库</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="42" hidden="0" customHeight="1">
@@ -7936,10 +7776,10 @@
         <x:v>铁氧化物逐级还原平衡</x:v>
       </x:c>
       <x:c r="D118" s="18" t="str">
-        <x:v>新增替换</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E118" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W18</x:v>
       </x:c>
       <x:c r="F118" s="18" t="str">
         <x:v>扩展</x:v>
@@ -7951,7 +7791,7 @@
         <x:v>高炉低碳</x:v>
       </x:c>
       <x:c r="I118" s="18" t="str">
-        <x:v>公式+既有热力学资产</x:v>
+        <x:v>PostgreSQL只读NIST/JANAF分段Shomate数据；500至1100 K</x:v>
       </x:c>
       <x:c r="J118" s="18" t="str">
         <x:v>否</x:v>
@@ -7960,10 +7800,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L118" s="18" t="str">
-        <x:v>metallurgy.extension.e022.v1</x:v>
+        <x:v>metallurgy.extension.e022.iron_oxide_step_reduction.v1</x:v>
       </x:c>
       <x:c r="M118" s="18" t="str">
-        <x:v>区别E002总铁平衡：E022给出各级热力学边界</x:v>
+        <x:v>Fe2O3→Fe3O4→FeO→Fe的CO/H2平衡；数据库缺失时关闭式失败</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="42" hidden="0" customHeight="1">
@@ -7974,13 +7814,13 @@
         <x:v>H001</x:v>
       </x:c>
       <x:c r="C119" s="18" t="str">
-        <x:v>钢液脱氧平衡</x:v>
+        <x:v>显式参数钢液脱氧平衡</x:v>
       </x:c>
       <x:c r="D119" s="18" t="str">
-        <x:v>新增替换</x:v>
+        <x:v>已实现</x:v>
       </x:c>
       <x:c r="E119" s="18" t="str">
-        <x:v>待分波实施</x:v>
+        <x:v>P1-W18</x:v>
       </x:c>
       <x:c r="F119" s="18" t="str">
         <x:v>扩展</x:v>
@@ -7992,7 +7832,7 @@
         <x:v>炉外精炼与洁净钢</x:v>
       </x:c>
       <x:c r="I119" s="18" t="str">
-        <x:v>公式+显式参数</x:v>
+        <x:v>调用方显式K或ΔG及Wagner项；PostgreSQL只读IUPAC原子量</x:v>
       </x:c>
       <x:c r="J119" s="18" t="str">
         <x:v>否</x:v>
@@ -8001,10 +7841,10 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="L119" s="18" t="str">
-        <x:v>metallurgy.extension.h001.v1</x:v>
+        <x:v>metallurgy.extension.h001.explicit_wagner_deoxidation.v1</x:v>
       </x:c>
       <x:c r="M119" s="18" t="str">
-        <x:v>新增炉外精炼能力；区别A007通用氧当量</x:v>
+        <x:v>Al/Si/Mn脱氧平衡；不臆造反应常数、交互参数、收得率或夹杂动力学</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="42" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
feat(platform): integrate tool orchestration and literature services
</commit_message>
<xml_diff>
--- a/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
+++ b/outputs/ds042_independent_replacement_plan_20260901/无现场数据依赖_120工具替换清单.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R31f7ef06e1544f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="Raf39284d2c784b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留5" sheetId="3" r:id="R2846b9a4e8b94a73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R202a3b95e8db4d14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="Rcd638e61da50497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R30cd5b42693a44a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="延期项20" sheetId="2" r:id="Rd3f0d543158448b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后续保留5" sheetId="3" r:id="R567d7fb8145d4271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增替换14" sheetId="4" r:id="R2470d92df4bb4d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终120路线" sheetId="5" r:id="R031d455e3d214665"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2072,7 +2072,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0b21bb605dc4b34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6270a8b02eec44a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7053,7 +7053,7 @@
         <x:v>仿真/优化/智能体支撑</x:v>
       </x:c>
       <x:c r="I100" s="18" t="str">
-        <x:v>显式长方体几何、网格、扩散率、边界与时间设置；仅生成OpenFOAM v13清单</x:v>
+        <x:v>显式长方体几何、网格、扩散率、边界与时间设置；可返回清单或在项目固定目录生成真实OpenFOAM v13案例与ZIP</x:v>
       </x:c>
       <x:c r="J100" s="18" t="str">
         <x:v>否</x:v>
@@ -7065,7 +7065,7 @@
         <x:v>metallurgy.catalog.g005.openfoam_laplacian_case.v1</x:v>
       </x:c>
       <x:c r="M100" s="18" t="str">
-        <x:v>受限laplacianFoam案例清单；不写任意路径、不执行求解器</x:v>
+        <x:v>受限laplacianFoam案例资产；固定目录落盘、回读校验、同名冲突拒绝；不执行求解器</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="42" hidden="0" customHeight="1">

</xml_diff>